<commit_message>
Updated behavior and solution approach with newly communicated design concerns. Refactoring.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Requirements/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D1F5A1-6565-8C41-9E32-37E112B5AD88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39BF9153-FC24-0C4F-9C79-95E34F8CC861}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5260" yWindow="780" windowWidth="30580" windowHeight="19500" activeTab="2" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="5260" yWindow="780" windowWidth="30580" windowHeight="19500" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="SoftwareRequirements" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Update to requirements to refine model of work and  account for the Zone Violation Computer model.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F92517FF-676B-D24A-A667-65932CD7874D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A3F999-C5FD-E445-8AEC-CBAEE42C94A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2000" yWindow="1840" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="262">
   <si>
     <t>Name</t>
   </si>
@@ -486,42 +486,15 @@
     <t>The zone alert service shall emit, as a message/event, each computed existing and imminent zone alert violation</t>
   </si>
   <si>
-    <t>SR-8-5-1</t>
-  </si>
-  <si>
     <t>The zone alert service shall emit each computed existing or imminent zone violation as a separate message/event</t>
   </si>
   <si>
-    <t>SR-8-5-2</t>
-  </si>
-  <si>
     <t>Each zone alert message/event shall indicate the vehicle ID of the vehicle to which the alert pertains</t>
   </si>
   <si>
     <t>Each zone alert message/event shall indicate the merged zone ID of the merged zone to which the alert pertains</t>
   </si>
   <si>
-    <t>SR-8-5-3</t>
-  </si>
-  <si>
-    <t>SR-8-5-4</t>
-  </si>
-  <si>
-    <t>SR-8-5-4-1</t>
-  </si>
-  <si>
-    <t>SR-8-5-4-2</t>
-  </si>
-  <si>
-    <t>SR-8-5-5</t>
-  </si>
-  <si>
-    <t>SR-8-5-5-1</t>
-  </si>
-  <si>
-    <t>SR-8-5-5-2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Each zone alert message/event shall report the time of the computed violation </t>
   </si>
   <si>
@@ -534,9 +507,6 @@
     <t>Each zone alert message shall indicate the time of an imminent zone volation as the time at which the predicted future violation is computed to first occur where the immediate previous time does not violate the zone</t>
   </si>
   <si>
-    <t>SR-8-5-6</t>
-  </si>
-  <si>
     <t>Each zone alert message/event shall indicate the position of an imminent zone volation as the position at which the future violation is computed to first occur where the immediate previous position does not violate the zone</t>
   </si>
   <si>
@@ -546,72 +516,36 @@
     <t>Each zone alert message/event shall indicate a time at which the computation of the particular alert occurred</t>
   </si>
   <si>
-    <t>The find first keep in zone function will determine if a received vehicle state report is the first one received for that vehicle, and if it is, determine the merged keep-in zone, if any, that the position is in or on the zone's polyhedron.</t>
-  </si>
-  <si>
-    <t>SR-8-7</t>
-  </si>
-  <si>
     <t>The zone alert service shall listen for and respond to each and every vehicle state messages/events by attempting to compute existing and imminent zone violations between the vehicle and each member of the set of  merged zones</t>
   </si>
   <si>
-    <t>The zone alert service shall compute whether an existing violation exists between a vehicle state and a merged zone</t>
-  </si>
-  <si>
     <t>SR-8-3-1</t>
   </si>
   <si>
-    <t>The zone alert service shall compute whether an existing violation exists between a vehicle state and a merged keep-out zone by determining whether the vehicle stated position is on or within the merged keep-out zone polyhedron.</t>
-  </si>
-  <si>
-    <t>The zone alert service shall compute whether an existing violation exists between a vehicle state and a merged keep-in zone by determining whether the merged keep-in zone is the original keep-in zone that the vehicle was in and whether the vehicle stated position is not in nor on the merged keep-in zone polyhedron.</t>
-  </si>
-  <si>
     <t>SR-8-3-2</t>
   </si>
   <si>
     <t>SR-8-3-2-1</t>
   </si>
   <si>
-    <t>The zone alert service shall determine and remember whether the first state report received for a vehicle is inside a merged keep-in zone and what that merged keep-in zone's id is.</t>
-  </si>
-  <si>
     <t>SR-8-4-1</t>
   </si>
   <si>
-    <t>The zone alert service shall compute the immediate linear trajectory line segment as the parametric line segment starting at but not including the vehicle's stated position at the stated time, along the vehicle's stated immediate velocity vector, to and including the position at the vehicle's stated time plus the services time window parameter.</t>
-  </si>
-  <si>
     <t>SR-8-4-2</t>
   </si>
   <si>
     <t>SR-8-4-3</t>
   </si>
   <si>
-    <t>The zone alert service shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-out zone by computing whether any point of the linear trajectory vector is on or in the merged keep-out zone's polyhedron</t>
-  </si>
-  <si>
     <t>SR-8-4-4</t>
   </si>
   <si>
-    <t>The zone alert service shall compute whether an imminent zone violation exists between a vehicle state and a merged zone</t>
-  </si>
-  <si>
     <t>The zone alert system shall emit no alert violations for undetermined violations</t>
   </si>
   <si>
     <t>SR-8-4-4-1</t>
   </si>
   <si>
-    <t xml:space="preserve">The zone alert service shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-in zone by computing if and only if the merged keep-in zone is the keep-in zone in which the first vehicle state report for the particular vehicle was in and any point of the linear trajectory vector is outside of the keep-out zone's polyhedron </t>
-  </si>
-  <si>
-    <t>The zone alert service shall compute whether an imminent zone violation exists between a vehicle state and a merged zone by computing if an existing zone violation does not exist between the vehicle state and merged zone and if the immediate linear trajectory of the vehicle state violates the merged zone</t>
-  </si>
-  <si>
-    <t>The zone alert service shall compute the position and time of an imminent zone volation as the position and time at which the future violation is computed to first occur where the immediate previous position does not violate the zone</t>
-  </si>
-  <si>
     <t>SR-8-4-5</t>
   </si>
   <si>
@@ -735,14 +669,170 @@
     <t>SR-7-6-6</t>
   </si>
   <si>
-    <t xml:space="preserve">The zone alert service shall call the zone alert computer to compute </t>
+    <t>SR-8-3-3-1</t>
+  </si>
+  <si>
+    <t>The zone alert service shall call the zone alert computer to compute  zone alerts against merged zones</t>
+  </si>
+  <si>
+    <t>SR-8-4-4-2</t>
+  </si>
+  <si>
+    <t>SR-8-4-5-1</t>
+  </si>
+  <si>
+    <t>SR-8-4-5-2</t>
+  </si>
+  <si>
+    <t>SR-8-4-6</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute/return all and only zone alerts between the provided vehicle state and the merged zones</t>
+  </si>
+  <si>
+    <t>SR-8-3-3</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute existing zone violation between a vehicle state and keep-out zone as the vehicle state's reported vehicle position being inside or on the keep-out zone polyhedron</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute imminent zone violation between a vehicle state and keep-out zone as the vehicle state's implied linear trajectory having one or more positions on or inside the keep-out zone's polyhedron</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute existing zone violation between a vehicle state and keep-in zone as the vehicle represented by the vehicle state having had an initial keep-in zone and the vehicle state reports's vehicle position being outside that implied keep-in zones polyhedron</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The implied merged keep-in zone of a vehicle will be the merged keep in zone that the vehicle's first received reported position (by vehicle state report) resides in or on the polyhedron of the merged keep-in zone, if any. </t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute imminent zone violation between a vehicle state and merged keep-in zone as the vehicle having the zone as its impled merged keep-in zone and the implied linear trajectory of the vehicle's received vehicle state having one or more points outside of the implied merged keep-in zone.</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute the implied linear trajectory of a vehicle state report as as the parametric line segment starting at but not including the vehicle's stated position at the stated time in the state report, along the vehicle's stated immediate velocity vector in the vehicle state report, to and including the position at the stated time in the vehicle state report plus the service's time window parameter.</t>
+  </si>
+  <si>
+    <t>BasicZoneAlertComputer</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-2</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-3</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-4</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-5</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-6</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall implement the zone alert computer</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-2</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-out zone by determining whether the vehicle stated position is on or within the merged keep-out zone polyhedron.</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-3</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute violation between a given vehicle state and merged zone by first computing whether the vehicle state is in existing violation with the zone, and if not, then computing whether the vehicle state is in imminent violation with the zone</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-7</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute the position and time of a detected imminent zone violation between the computed immediate trajectory vector and the keep-in zone as the first time and position in the parametric trajectory on the surface of the polyhedron where the temporally next trajectory positions are outside the polyherdron.</t>
+  </si>
+  <si>
+    <t>SR-8-3-2-8</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall compute the position and time of a detected existing zone violation between a vehicle's stated position and a merged zone as the stated vehicle position and time of the vehicle state report.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-in zone by determining whether the merged keep-in zone is the original keep-in zone that the vehicle was in and whether the vehicle stated position is not in nor on the merged keep-in zone polyhedron.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall determine whether the vehicle state report is the first such received report for a given vehicle id</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute for each vehicle whose state reports are received the implied keep-in zone for the vehicle</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall, if it has received the first vehicle state report for a given vehicle id, which if any merged keep-in zone the reported vehicle position of the state report resides in or on.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute, for each merged keep-in zone, whether a given position is in or on the zone</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-4</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-4-1</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-4-2</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-4-3</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-4-4</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall record the association between the vehicle and merged keep-in zone in or on which the vehicle's first stated position is found</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-5</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-5-1</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-5-2</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-5-2-1</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-5-3</t>
+  </si>
+  <si>
+    <t>SR-8-3-3-3-3-1</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether an imminent zone violation exists between a vehicle state and a merged zone by computing if an existing zone violation does not exist between the vehicle state and merged zone and if the immediate linear trajectory of the vehicle state violates the merged zone</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute the immediate linear trajectory line segment as the parametric line segment starting at but not including the vehicle's stated position at the stated time, along the vehicle's stated immediate velocity vector, to and including the position at the vehicle's stated time plus the services time window parameter.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-out zone by computing whether any point of the linear trajectory vector is on or in the merged keep-out zone's polyhedron</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-out zone as the first time and position in the parametric trajectory on the surface of the polyhedron where the temporally next trajectory positions are inside the polyherdron.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-in zone by computing if and only if the merged keep-in zone is the zone associated with the vehicle id found in the vehicle's first state report and (short-circuit) and any point of the linear trajectory vector is outside of the keep-in zone's polyhedron </t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-in zone as the first time and position in the parametric trajectory on the surface of the polyhedron where the temporally next trajectory positions are outside the polyhedron.</t>
+  </si>
+  <si>
+    <t>The zone alert service shall respond to a received vehicle state by computing whether a violation exists between the received vehicle state and each merged zone as defined by its polygedral boundary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -783,6 +873,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -874,7 +971,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
@@ -911,6 +1008,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -1255,7 +1353,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34AC7C05-FC71-F749-BB41-F1A5141E29DB}">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -1279,7 +1377,7 @@
         <v>91</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>191</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.2">
@@ -1293,7 +1391,7 @@
         <v>79</v>
       </c>
       <c r="E2" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1304,40 +1402,40 @@
         <v>78</v>
       </c>
       <c r="E3" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>194</v>
+        <v>172</v>
       </c>
       <c r="E4" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="E5" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>195</v>
+        <v>173</v>
       </c>
       <c r="E6" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1351,29 +1449,29 @@
         <v>81</v>
       </c>
       <c r="E7" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
       <c r="E8" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
       <c r="E9" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1384,7 +1482,7 @@
         <v>93</v>
       </c>
       <c r="E10" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1395,7 +1493,7 @@
         <v>94</v>
       </c>
       <c r="E11" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1406,29 +1504,29 @@
         <v>95</v>
       </c>
       <c r="E12" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="E13" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="E14" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1442,7 +1540,7 @@
         <v>90</v>
       </c>
       <c r="E15" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1453,7 +1551,7 @@
         <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1464,7 +1562,7 @@
         <v>98</v>
       </c>
       <c r="E17" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1475,29 +1573,29 @@
         <v>99</v>
       </c>
       <c r="E18" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="E19" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="E20" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1508,7 +1606,7 @@
         <v>102</v>
       </c>
       <c r="E21" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1519,7 +1617,7 @@
         <v>104</v>
       </c>
       <c r="E22" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1530,7 +1628,7 @@
         <v>107</v>
       </c>
       <c r="E23" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1538,10 +1636,10 @@
         <v>108</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="E24" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1552,18 +1650,18 @@
         <v>113</v>
       </c>
       <c r="E25" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="E26" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1574,29 +1672,29 @@
         <v>109</v>
       </c>
       <c r="E27" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>221</v>
+        <v>199</v>
       </c>
       <c r="E28" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>220</v>
+        <v>198</v>
       </c>
       <c r="E29" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1607,29 +1705,29 @@
         <v>110</v>
       </c>
       <c r="E30" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>222</v>
+        <v>200</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>223</v>
+        <v>201</v>
       </c>
       <c r="E31" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="E32" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1640,7 +1738,7 @@
         <v>122</v>
       </c>
       <c r="E33" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1651,7 +1749,7 @@
         <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1662,7 +1760,7 @@
         <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1673,7 +1771,7 @@
         <v>126</v>
       </c>
       <c r="E36" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1684,7 +1782,7 @@
         <v>123</v>
       </c>
       <c r="E37" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1695,7 +1793,7 @@
         <v>125</v>
       </c>
       <c r="E38" t="s">
-        <v>224</v>
+        <v>202</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1706,7 +1804,7 @@
         <v>111</v>
       </c>
       <c r="E39" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1717,7 +1815,7 @@
         <v>112</v>
       </c>
       <c r="E40" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1728,7 +1826,7 @@
         <v>131</v>
       </c>
       <c r="E41" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1736,10 +1834,10 @@
         <v>132</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>225</v>
+        <v>203</v>
       </c>
       <c r="E42" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1747,10 +1845,10 @@
         <v>134</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E43" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1758,43 +1856,43 @@
         <v>137</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="E44" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>226</v>
+        <v>204</v>
       </c>
       <c r="C45" s="13" t="s">
         <v>133</v>
       </c>
       <c r="E45" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
       <c r="C46" s="13" t="s">
         <v>135</v>
       </c>
       <c r="E46" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>230</v>
+        <v>208</v>
       </c>
       <c r="C47" s="13" t="s">
         <v>136</v>
       </c>
       <c r="E47" t="s">
-        <v>227</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="34" x14ac:dyDescent="0.2">
@@ -1805,10 +1903,10 @@
         <v>139</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="E48" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1819,7 +1917,7 @@
         <v>141</v>
       </c>
       <c r="E49" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1830,7 +1928,7 @@
         <v>143</v>
       </c>
       <c r="E50" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="17" x14ac:dyDescent="0.2">
@@ -1838,268 +1936,407 @@
         <v>144</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>171</v>
+        <v>261</v>
       </c>
       <c r="E51" t="s">
-        <v>192</v>
+        <v>170</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>210</v>
+      </c>
+      <c r="E52" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+      <c r="E53" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+      <c r="E54" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>176</v>
+        <v>224</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+      <c r="E55" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>145</v>
+        <v>225</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>184</v>
+        <v>220</v>
+      </c>
+      <c r="E56" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>178</v>
+      <c r="A57" s="18" t="s">
+        <v>226</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>188</v>
+        <v>218</v>
+      </c>
+      <c r="E57" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>180</v>
+      <c r="A58" s="18" t="s">
+        <v>227</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>181</v>
+        <v>221</v>
+      </c>
+      <c r="E58" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+      <c r="A59" s="18" t="s">
+        <v>228</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>182</v>
+        <v>222</v>
+      </c>
+      <c r="E59" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>183</v>
+      <c r="A60" s="18" t="s">
+        <v>234</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>187</v>
+        <v>237</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>229</v>
+      </c>
+      <c r="E62" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>146</v>
+        <v>209</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>148</v>
+        <v>230</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>150</v>
+        <v>232</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>151</v>
+        <v>238</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>153</v>
+        <v>243</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>152</v>
+        <v>240</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>154</v>
+        <v>244</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>160</v>
+        <v>239</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>155</v>
+        <v>245</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>156</v>
+        <v>246</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>163</v>
+        <v>242</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>157</v>
+        <v>247</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>158</v>
+        <v>249</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>166</v>
+        <v>255</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>159</v>
+        <v>250</v>
       </c>
       <c r="C72" s="13" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>251</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>252</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>253</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>254</v>
+      </c>
+      <c r="C76" s="13" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>145</v>
+      </c>
+      <c r="C77" s="13" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>162</v>
+      </c>
+      <c r="C78" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>163</v>
+      </c>
+      <c r="C79" s="13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>164</v>
+      </c>
+      <c r="C80" s="13" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>164</v>
-      </c>
-      <c r="C73" s="13" t="s">
+      <c r="C81" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="17" x14ac:dyDescent="0.2">
-      <c r="A74" t="s">
-        <v>169</v>
-      </c>
-      <c r="C74" s="13" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C75" s="13"/>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C76" s="13"/>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C77" s="13"/>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C78" s="13"/>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C79" s="13"/>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C80" s="13"/>
-    </row>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C81" s="13"/>
-    </row>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C82" s="14"/>
-    </row>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C83" s="14"/>
-    </row>
-    <row r="84" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C84" s="14"/>
-    </row>
-    <row r="85" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C85" s="13"/>
-    </row>
-    <row r="86" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C86" s="14"/>
-    </row>
-    <row r="87" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C87" s="14"/>
-    </row>
-    <row r="88" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C88" s="14"/>
-    </row>
-    <row r="89" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C89" s="14"/>
-    </row>
-    <row r="90" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C90" s="14"/>
-      <c r="D90" s="13"/>
-    </row>
-    <row r="91" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C82" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>211</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>168</v>
+      </c>
+      <c r="C84" s="13" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>212</v>
+      </c>
+      <c r="C85" s="13" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>213</v>
+      </c>
+      <c r="C86" s="13" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>214</v>
+      </c>
+      <c r="C87" s="13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>146</v>
+      </c>
+      <c r="C88" s="13" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C89" s="13"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C90" s="13"/>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C91" s="13"/>
     </row>
-    <row r="92" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C92" s="14"/>
-    </row>
-    <row r="93" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C93" s="14"/>
-    </row>
-    <row r="94" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C94" s="14"/>
-    </row>
-    <row r="95" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C95" s="14"/>
-    </row>
-    <row r="96" spans="3:4" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C92" s="13"/>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C93" s="13"/>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C94" s="13"/>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C95" s="13"/>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C96" s="14"/>
     </row>
-    <row r="97" spans="3:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C97" s="14"/>
     </row>
-    <row r="98" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C98" s="13"/>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C98" s="14"/>
+    </row>
+    <row r="99" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C99" s="13"/>
+    </row>
+    <row r="100" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C100" s="14"/>
+    </row>
+    <row r="101" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C101" s="14"/>
+    </row>
+    <row r="102" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C102" s="14"/>
+    </row>
+    <row r="103" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C103" s="14"/>
+    </row>
+    <row r="104" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C104" s="14"/>
+      <c r="D104" s="13"/>
+    </row>
+    <row r="105" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C105" s="13"/>
+    </row>
+    <row r="106" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C106" s="14"/>
+    </row>
+    <row r="107" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C107" s="14"/>
+    </row>
+    <row r="108" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C108" s="14"/>
+    </row>
+    <row r="109" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C109" s="14"/>
+    </row>
+    <row r="110" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C110" s="14"/>
+    </row>
+    <row r="111" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C111" s="14"/>
+    </row>
+    <row r="112" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C112" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated specifications to assume 2D merged zone semantics for detection of zone violations.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7A3F999-C5FD-E445-8AEC-CBAEE42C94A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA5F7A8A-1049-9F45-BEBE-DC04E9BA0A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2000" yWindow="1840" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="900" yWindow="1100" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="TopLevelRequirements" sheetId="6" r:id="rId1"/>
     <sheet name="SolutionRequirements" sheetId="4" r:id="rId2"/>
-    <sheet name="SoftwareRequirements" sheetId="1" r:id="rId3"/>
-    <sheet name="Interface Def and Reqs" sheetId="3" r:id="rId4"/>
-    <sheet name="Requiremnts Unknowns" sheetId="2" r:id="rId5"/>
+    <sheet name="Interface Def and Reqs" sheetId="3" r:id="rId3"/>
+    <sheet name="Requiremnts Unknowns" sheetId="2" r:id="rId4"/>
+    <sheet name="OLD SoftwareRequirements" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="266">
   <si>
     <t>Name</t>
   </si>
@@ -261,15 +261,9 @@
     <t>HL-1</t>
   </si>
   <si>
-    <t>Provide  an OpenUxAS service to make OpenUxAS systems aware of existing zone violations by vehicles</t>
-  </si>
-  <si>
     <t>Provide an OpenUxAS service to make OpenUxAS systems aware of potential for future zone violations by vehicles based on zone and vehicle positinos and vehicle behavior</t>
   </si>
   <si>
-    <t>HL-2</t>
-  </si>
-  <si>
     <t>CATEGORY</t>
   </si>
   <si>
@@ -285,9 +279,6 @@
     <t>Service Preparation and Listening Phase</t>
   </si>
   <si>
-    <t>The service shall begin by listening for and recording information about the OpenUxAS missions environment and actors</t>
-  </si>
-  <si>
     <t>SR-1</t>
   </si>
   <si>
@@ -384,18 +375,12 @@
     <t>The service shall perform zone merging  on the zones declared by other OpenUxAS message senders</t>
   </si>
   <si>
-    <t>SR-7-3-1</t>
-  </si>
-  <si>
     <t>SR-7</t>
   </si>
   <si>
     <t>SR-7-2</t>
   </si>
   <si>
-    <t>SR-7-3</t>
-  </si>
-  <si>
     <t>SR-7-4</t>
   </si>
   <si>
@@ -405,57 +390,18 @@
     <t>SR-7-6</t>
   </si>
   <si>
-    <t xml:space="preserve">The zone merging function shall take as input all declared zones, each a polyhedra in Cartesian space, and output the merged zones, each as a polyhedra in Cartesian space </t>
-  </si>
-  <si>
-    <t xml:space="preserve">The zone merging function shall satisfy the intent of merging an input set of zones into a set of zones such that any overlapping zones of the same type are now part of the same zoneat is the spatial cover, with holes removed, each representing sets of zones that overlap in Caretesian space into a single zone. </t>
-  </si>
-  <si>
-    <t>The zone merging function shall merge overlapping zones in the x-y plane with the same semantics of the prefered OpenUxAS Route Planning service</t>
-  </si>
-  <si>
-    <t>The zone merging function  shall perform zone merging that satisfies, to the extent possible in 3 dimensions, the zone merging semantics of the prefered OpenUxAS route planning service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The zone merging functional shall merge altitude bounds merged zones by choosing the tightest altitude bounds that contain altitude bounds of its input overlapping zones </t>
-  </si>
-  <si>
-    <t>The merging function shall not merge any zones that are not of the same type where type is keep-in or keep-out.</t>
-  </si>
-  <si>
-    <t>SR-7-3-2</t>
-  </si>
-  <si>
-    <t>SR-7-3-2-1</t>
-  </si>
-  <si>
-    <t>SR-7-3-2-2</t>
-  </si>
-  <si>
-    <t>SR-7-3-2-3</t>
-  </si>
-  <si>
     <t>The service shall announce each merged zone by emitting the merged zone as a declaration message/event in OpenUxAS</t>
   </si>
   <si>
-    <t>SR-7-6-1</t>
-  </si>
-  <si>
     <t>Each merged zone declaration message/event shall state the assigned ID of the merged zone</t>
   </si>
   <si>
-    <t>SR-7-6-2</t>
-  </si>
-  <si>
     <t>Each merged zone declaration message/event shall state the geometry of the merged zone polyhedron</t>
   </si>
   <si>
     <t>Each merged zone declaration message/event shall state whether the merged zone is keep-out or keep-in</t>
   </si>
   <si>
-    <t>SR-7-6-3</t>
-  </si>
-  <si>
     <t>SR-8</t>
   </si>
   <si>
@@ -561,9 +507,6 @@
     <t>The service shall initiate by creating and installing a ZoneAlertComputer</t>
   </si>
   <si>
-    <t>The installed ZoneAlertComputer shall determine whether a given time window is acceptable to it</t>
-  </si>
-  <si>
     <t>The service shall create and install one and only one  ZoneAlertComputer</t>
   </si>
   <si>
@@ -576,9 +519,6 @@
     <t>The zone alert service shall pass received vehicle declarations to its ZoneAlertCompter</t>
   </si>
   <si>
-    <t>The zone alert service shall pass received zone declarations to its ZoneAlertCompter</t>
-  </si>
-  <si>
     <t>SR-4-2-1</t>
   </si>
   <si>
@@ -654,21 +594,12 @@
     <t>The Zone Alert Computer mergeZones function shall return the sets of created merged zones, both keep-in and keep-out, providing a merged zone's id and its full geometry for each and every such created merged zone</t>
   </si>
   <si>
-    <t>SR-7-6-4</t>
-  </si>
-  <si>
     <t>ZoneAlertService, CMASI</t>
   </si>
   <si>
     <t>The Zone Alert Service shall take the set of returned merged keep-in zones and announce each and every one as a Merged Zone Declarations to OpenUxAS as OpenUxAS event/messages</t>
   </si>
   <si>
-    <t>SR-7-6-5</t>
-  </si>
-  <si>
-    <t>SR-7-6-6</t>
-  </si>
-  <si>
     <t>SR-8-3-3-1</t>
   </si>
   <si>
@@ -735,9 +666,6 @@
     <t>SR-8-3-3-2</t>
   </si>
   <si>
-    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-out zone by determining whether the vehicle stated position is on or within the merged keep-out zone polyhedron.</t>
-  </si>
-  <si>
     <t>SR-8-3-3-3</t>
   </si>
   <si>
@@ -756,9 +684,6 @@
     <t>The zone alert computer shall compute the position and time of a detected existing zone violation between a vehicle's stated position and a merged zone as the stated vehicle position and time of the vehicle state report.</t>
   </si>
   <si>
-    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-in zone by determining whether the merged keep-in zone is the original keep-in zone that the vehicle was in and whether the vehicle stated position is not in nor on the merged keep-in zone polyhedron.</t>
-  </si>
-  <si>
     <t>The basic zone alert computer shall determine whether the vehicle state report is the first such received report for a given vehicle id</t>
   </si>
   <si>
@@ -768,9 +693,6 @@
     <t>The basic zone alert computer shall, if it has received the first vehicle state report for a given vehicle id, which if any merged keep-in zone the reported vehicle position of the state report resides in or on.</t>
   </si>
   <si>
-    <t>The basic zone alert computer shall compute, for each merged keep-in zone, whether a given position is in or on the zone</t>
-  </si>
-  <si>
     <t>SR-8-3-3-4</t>
   </si>
   <si>
@@ -813,19 +735,109 @@
     <t>The basic zone alert computer shall compute the immediate linear trajectory line segment as the parametric line segment starting at but not including the vehicle's stated position at the stated time, along the vehicle's stated immediate velocity vector, to and including the position at the vehicle's stated time plus the services time window parameter.</t>
   </si>
   <si>
-    <t>The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-out zone by computing whether any point of the linear trajectory vector is on or in the merged keep-out zone's polyhedron</t>
-  </si>
-  <si>
-    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-out zone as the first time and position in the parametric trajectory on the surface of the polyhedron where the temporally next trajectory positions are inside the polyherdron.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-in zone by computing if and only if the merged keep-in zone is the zone associated with the vehicle id found in the vehicle's first state report and (short-circuit) and any point of the linear trajectory vector is outside of the keep-in zone's polyhedron </t>
-  </si>
-  <si>
-    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-in zone as the first time and position in the parametric trajectory on the surface of the polyhedron where the temporally next trajectory positions are outside the polyhedron.</t>
-  </si>
-  <si>
     <t>The zone alert service shall respond to a received vehicle state by computing whether a violation exists between the received vehicle state and each merged zone as defined by its polygedral boundary</t>
+  </si>
+  <si>
+    <t>The service shal utilize the same semantics for zone geometry as route planning service</t>
+  </si>
+  <si>
+    <t>OpenUxAS shall be aware of existing zone violations by vehicles to usefully avoiid/recover/accept imminent and existing zone violations.</t>
+  </si>
+  <si>
+    <t>HL-1-1</t>
+  </si>
+  <si>
+    <t>HL-1-2</t>
+  </si>
+  <si>
+    <t>SR-3.1.1</t>
+  </si>
+  <si>
+    <t>The service shall proceed initialization on parameters by by listening for and recording information about the OpenUxAS missions environment and actors</t>
+  </si>
+  <si>
+    <t>The zone alert service shall pass each received zone declarations to its ZoneAlertComputer</t>
+  </si>
+  <si>
+    <t>The zone alert sevice</t>
+  </si>
+  <si>
+    <t>The installed ZoneAlertComputer shall determine whether a given time window is acceptable to it to be able to effectivel compute imminent zone alerts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Authoritative Zone Merging Model shall merge all zones such that all zones of the same type (keep-in or keep-out) are merged into a single zone with each and every zone of the same type with which they overlap or touch in the horizontal plane. </t>
+  </si>
+  <si>
+    <t>The Authoritative Zone Merging Model shall merge all zones such that all zones conserve their initial encompassed area in the horizontal plane.</t>
+  </si>
+  <si>
+    <t>The Authoritative Zone Merging Model shall merge zones shall allow internal holes that are created in the merging of a zone to be ignored, including that area in the resulting merged zones in the horizontal plane</t>
+  </si>
+  <si>
+    <t>The Authoritative Zone Merging Model shall not create geometry in the vertical plane, with the assumption that all altitudes are included in the merged zone semantics.</t>
+  </si>
+  <si>
+    <t>The zone merging function shall satisty the intent of taking as input the set of all declared zones and producing as output merged zones satisfing the Authoritative Zone Merging Model</t>
+  </si>
+  <si>
+    <t>The Authoritative Zone Merging Model shall merge overlapping zones in the x-y plane with the same semantics of the prefered OpenUxAS Route Planning service</t>
+  </si>
+  <si>
+    <t>SR-7-2-3</t>
+  </si>
+  <si>
+    <t>SR-7-2-3-1</t>
+  </si>
+  <si>
+    <t>SR-7-2-3-2</t>
+  </si>
+  <si>
+    <t>SR-7-2-3-3</t>
+  </si>
+  <si>
+    <t>SR-7-3-3-4</t>
+  </si>
+  <si>
+    <t>SR-7-7</t>
+  </si>
+  <si>
+    <t>SR-7-7-1</t>
+  </si>
+  <si>
+    <t>SR-7-7-2</t>
+  </si>
+  <si>
+    <t>SR-7-7-3</t>
+  </si>
+  <si>
+    <t>SR-7-7-4</t>
+  </si>
+  <si>
+    <t>SR-7-7-5</t>
+  </si>
+  <si>
+    <t>SR-7-7-6</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-out zone by determining whether the vehicle stated position is on or within the merged keep-out zone polygon in the horizontal plane.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether an existing violation exists between a vehicle state and a merged keep-in zone by determining whether the merged keep-in zone is the original keep-in zone that the vehicle was in and whether the vehicle stated position is not in nor on the merged keep-in zone polygon in the x-y plane.</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute, for each merged keep-in zone, whether a given position is in or on the zone's polygon boundary in the x-y plane</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-out zone by computing whether any point of the linear trajectory vector is on or in the merged keep-out zone's polygon boundary in the x-y plane</t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-out zone as the first time and position in the parametric trajectory on the edges (and vertices) of the polygon in the horizontal plane where the temporally next trajectory positions are inside the polygon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The basic zone alert computer shall compute whether a vehicle state's computed immediate trajectory vector violates a merged keep-in zone by computing if and only if the merged keep-in zone is the zone associated with the vehicle id found in the vehicle's first state report and (short-circuit) and any point of the linear trajectory vector is outside of the keep-in zone's polygon </t>
+  </si>
+  <si>
+    <t>The basic zone alert computer shall compute the position and time of the imminent zone violation between the computed immediate trajectory vector and the keep-in zone as the first time and position in the parametric trajectory on the edges (and vertices) of the polgon in the horizontal plane where the temporally next trajectory positions is outside the polygon in the horizontal plane.</t>
   </si>
 </sst>
 </file>
@@ -971,7 +983,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
@@ -1009,6 +1021,8 @@
       <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
@@ -1324,7 +1338,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FDF8AA6-5D75-9940-86F4-A0A21993176A}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="45.5" customWidth="1"/>
@@ -1335,15 +1349,23 @@
         <v>72</v>
       </c>
       <c r="B1" t="s">
-        <v>73</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>234</v>
       </c>
       <c r="B2" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B3" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -1353,7 +1375,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34AC7C05-FC71-F749-BB41-F1A5141E29DB}">
-  <dimension ref="A1:E112"/>
+  <dimension ref="A1:E113"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -1368,905 +1390,898 @@
         <v>70</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C1" s="11" t="s">
         <v>71</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>169</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>79</v>
-      </c>
       <c r="E2" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>172</v>
+        <v>154</v>
       </c>
       <c r="E4" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>174</v>
+        <v>155</v>
       </c>
       <c r="E5" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>180</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="E6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B7" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="13" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A6" s="20" t="s">
+        <v>160</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" s="20" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A7" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="E7" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>175</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="E8" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>176</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="E9" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="17" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>93</v>
-      </c>
-      <c r="E10" t="s">
-        <v>170</v>
+      <c r="B7" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" s="20" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A8" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A9" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" s="19" customFormat="1" ht="17" x14ac:dyDescent="0.2">
+      <c r="A10" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="19" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E11" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E12" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>179</v>
+        <v>84</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>183</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>184</v>
+        <v>163</v>
       </c>
       <c r="E14" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>165</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="D15" t="s">
-        <v>90</v>
+        <v>164</v>
       </c>
       <c r="E15" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>96</v>
+        <v>86</v>
+      </c>
+      <c r="D16" t="s">
+        <v>87</v>
       </c>
       <c r="E16" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>89</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E17" t="s">
-        <v>186</v>
+        <v>152</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>187</v>
+        <v>97</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>190</v>
+        <v>96</v>
       </c>
       <c r="E19" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="E20" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" s="15" t="s">
-        <v>102</v>
+        <v>168</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>169</v>
       </c>
       <c r="E21" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="E22" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="E23" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>191</v>
+        <v>104</v>
       </c>
       <c r="E24" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>113</v>
+        <v>171</v>
       </c>
       <c r="E25" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>193</v>
+        <v>111</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>192</v>
+        <v>110</v>
       </c>
       <c r="E26" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>173</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>109</v>
+        <v>172</v>
       </c>
       <c r="E27" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>194</v>
+        <v>100</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>199</v>
+        <v>106</v>
       </c>
       <c r="E28" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>196</v>
+        <v>174</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>198</v>
+        <v>179</v>
       </c>
       <c r="E29" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>116</v>
+        <v>176</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>110</v>
+        <v>178</v>
       </c>
       <c r="E30" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>200</v>
+        <v>112</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>201</v>
+        <v>107</v>
       </c>
       <c r="E31" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>197</v>
+        <v>181</v>
       </c>
       <c r="E32" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>175</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>122</v>
+        <v>177</v>
       </c>
       <c r="E33" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>114</v>
+        <v>247</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="E34" t="s">
-        <v>202</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>127</v>
-      </c>
-      <c r="C35" s="17" t="s">
-        <v>124</v>
-      </c>
-      <c r="E35" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>248</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>128</v>
-      </c>
-      <c r="C36" s="17" t="s">
-        <v>126</v>
-      </c>
-      <c r="E36" t="s">
-        <v>202</v>
+        <v>249</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>243</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>129</v>
+        <v>250</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="E37" t="s">
-        <v>202</v>
+        <v>244</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>130</v>
-      </c>
-      <c r="C38" s="16" t="s">
-        <v>125</v>
+        <v>251</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>246</v>
       </c>
       <c r="E38" t="s">
-        <v>202</v>
+        <v>182</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>111</v>
+        <v>245</v>
       </c>
       <c r="E39" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E40" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>120</v>
-      </c>
-      <c r="C41" s="13" t="s">
-        <v>131</v>
+        <v>115</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>109</v>
       </c>
       <c r="E41" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>132</v>
+        <v>252</v>
       </c>
       <c r="C42" s="13" t="s">
-        <v>203</v>
+        <v>116</v>
       </c>
       <c r="E42" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>134</v>
+        <v>253</v>
       </c>
       <c r="C43" s="13" t="s">
-        <v>206</v>
+        <v>183</v>
       </c>
       <c r="E43" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>137</v>
+        <v>254</v>
       </c>
       <c r="C44" s="13" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="E44" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>204</v>
+        <v>255</v>
       </c>
       <c r="C45" s="13" t="s">
-        <v>133</v>
+        <v>185</v>
       </c>
       <c r="E45" t="s">
-        <v>205</v>
+        <v>152</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>207</v>
+        <v>256</v>
       </c>
       <c r="C46" s="13" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="E46" t="s">
-        <v>205</v>
+        <v>184</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>208</v>
+        <v>257</v>
       </c>
       <c r="C47" s="13" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="E47" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>138</v>
-      </c>
-      <c r="B48" t="s">
-        <v>139</v>
+        <v>258</v>
       </c>
       <c r="C48" s="13" t="s">
-        <v>158</v>
+        <v>119</v>
       </c>
       <c r="E48" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
+        <v>120</v>
+      </c>
+      <c r="B49" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="C49" s="13" t="s">
-        <v>141</v>
-      </c>
       <c r="E49" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>142</v>
+        <v>122</v>
       </c>
       <c r="C50" s="13" t="s">
-        <v>143</v>
+        <v>123</v>
       </c>
       <c r="E50" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>144</v>
+        <v>124</v>
       </c>
       <c r="C51" s="13" t="s">
-        <v>261</v>
+        <v>125</v>
       </c>
       <c r="E51" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>159</v>
+        <v>126</v>
       </c>
       <c r="C52" s="13" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="E52" t="s">
-        <v>170</v>
+        <v>152</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>160</v>
+        <v>141</v>
       </c>
       <c r="C53" s="13" t="s">
-        <v>215</v>
+        <v>187</v>
       </c>
       <c r="E53" t="s">
-        <v>171</v>
+        <v>152</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="C54" s="13" t="s">
-        <v>217</v>
+        <v>192</v>
       </c>
       <c r="E54" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>224</v>
+        <v>143</v>
       </c>
       <c r="C55" s="13" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="E55" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>225</v>
+        <v>201</v>
       </c>
       <c r="C56" s="13" t="s">
-        <v>220</v>
+        <v>196</v>
       </c>
       <c r="E56" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A57" s="18" t="s">
-        <v>226</v>
+      <c r="A57" t="s">
+        <v>202</v>
       </c>
       <c r="C57" s="13" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="E57" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A58" s="18" t="s">
-        <v>227</v>
+        <v>203</v>
       </c>
       <c r="C58" s="13" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="E58" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" ht="51" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A59" s="18" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>222</v>
+        <v>198</v>
       </c>
       <c r="E59" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="51" x14ac:dyDescent="0.2">
       <c r="A60" s="18" t="s">
-        <v>234</v>
+        <v>205</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>237</v>
+        <v>199</v>
+      </c>
+      <c r="E60" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="34" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
-        <v>236</v>
+      <c r="A61" s="18" t="s">
+        <v>210</v>
       </c>
       <c r="C61" s="13" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C62" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="E62" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" ht="34" x14ac:dyDescent="0.2">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="17" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="C63" s="13" t="s">
-        <v>233</v>
+        <v>206</v>
+      </c>
+      <c r="E63" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>230</v>
+        <v>186</v>
       </c>
       <c r="C64" s="13" t="s">
-        <v>231</v>
+        <v>209</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>232</v>
+        <v>207</v>
       </c>
       <c r="C65" s="13" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="C66" s="13" t="s">
-        <v>240</v>
+        <v>260</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>244</v>
+        <v>217</v>
       </c>
       <c r="C67" s="13" t="s">
-        <v>239</v>
+        <v>215</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>245</v>
+        <v>218</v>
       </c>
       <c r="C68" s="13" t="s">
-        <v>241</v>
+        <v>214</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>246</v>
+        <v>219</v>
       </c>
       <c r="C69" s="13" t="s">
-        <v>242</v>
+        <v>216</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>247</v>
+        <v>220</v>
       </c>
       <c r="C70" s="13" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>249</v>
+        <v>221</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>255</v>
+        <v>222</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>250</v>
+        <v>223</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>256</v>
+        <v>229</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>251</v>
+        <v>224</v>
       </c>
       <c r="C73" s="13" t="s">
-        <v>257</v>
+        <v>230</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>252</v>
+        <v>225</v>
       </c>
       <c r="C74" s="13" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>253</v>
+        <v>226</v>
       </c>
       <c r="C75" s="13" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>254</v>
+        <v>227</v>
       </c>
       <c r="C76" s="13" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>145</v>
+        <v>228</v>
       </c>
       <c r="C77" s="13" t="s">
-        <v>147</v>
+        <v>265</v>
       </c>
     </row>
     <row r="78" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>162</v>
+        <v>127</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
     </row>
     <row r="79" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>163</v>
+        <v>144</v>
       </c>
       <c r="C79" s="13" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
     </row>
     <row r="80" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>164</v>
+        <v>145</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
     </row>
     <row r="81" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>165</v>
+        <v>146</v>
       </c>
       <c r="C81" s="13" t="s">
-        <v>151</v>
+        <v>132</v>
       </c>
     </row>
     <row r="82" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>167</v>
+        <v>147</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>211</v>
+        <v>149</v>
       </c>
       <c r="C83" s="13" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>168</v>
+        <v>188</v>
       </c>
       <c r="C84" s="13" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>212</v>
+        <v>150</v>
       </c>
       <c r="C85" s="13" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="34" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>213</v>
+        <v>189</v>
       </c>
       <c r="C86" s="13" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>214</v>
+        <v>190</v>
       </c>
       <c r="C87" s="13" t="s">
-        <v>157</v>
+        <v>137</v>
       </c>
     </row>
     <row r="88" spans="1:3" ht="17" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>146</v>
+        <v>191</v>
       </c>
       <c r="C88" s="13" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C89" s="13"/>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" ht="17" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>128</v>
+      </c>
+      <c r="C89" s="13" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="C90" s="13"/>
@@ -2287,7 +2302,7 @@
       <c r="C95" s="13"/>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="C96" s="14"/>
+      <c r="C96" s="13"/>
     </row>
     <row r="97" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C97" s="14"/>
@@ -2296,10 +2311,10 @@
       <c r="C98" s="14"/>
     </row>
     <row r="99" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C99" s="13"/>
+      <c r="C99" s="14"/>
     </row>
     <row r="100" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C100" s="14"/>
+      <c r="C100" s="13"/>
     </row>
     <row r="101" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C101" s="14"/>
@@ -2312,13 +2327,13 @@
     </row>
     <row r="104" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C104" s="14"/>
-      <c r="D104" s="13"/>
     </row>
     <row r="105" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C105" s="13"/>
+      <c r="C105" s="14"/>
+      <c r="D105" s="13"/>
     </row>
     <row r="106" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C106" s="14"/>
+      <c r="C106" s="13"/>
     </row>
     <row r="107" spans="3:4" x14ac:dyDescent="0.2">
       <c r="C107" s="14"/>
@@ -2336,7 +2351,10 @@
       <c r="C111" s="14"/>
     </row>
     <row r="112" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C112" s="13"/>
+      <c r="C112" s="14"/>
+    </row>
+    <row r="113" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C113" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2344,6 +2362,110 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3702B00E-AAB7-7F4B-9F1C-57A3CF73FDCB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA87E05-7BE7-9C44-A27E-E2FA4156C15F}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="36.83203125" style="3" customWidth="1"/>
+    <col min="2" max="2" width="95.33203125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="44.33203125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="43.83203125" style="5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="22" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="35" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="153" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="C8" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E717DA4B-5271-1F48-AA72-ACE0E1514F9D}">
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2606,108 +2728,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3702B00E-AAB7-7F4B-9F1C-57A3CF73FDCB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BA87E05-7BE7-9C44-A27E-E2FA4156C15F}">
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="36.83203125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="95.33203125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="44.33203125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="43.83203125" style="5" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" ht="22" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="35" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="B3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="51" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="153" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="C8" s="9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated issues and requirements to fix a lack of an important failed constraint to propagate from Hight Level to Software Level requirements.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED9DBE1-13B0-6D40-BF1F-63FF89C81251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D260B86-EAE2-F648-BE4C-5D50B132DA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="2" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
-    <sheet name="TopLevelRequirements" sheetId="6" r:id="rId1"/>
+    <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
     <sheet name="SolutionRequirements" sheetId="4" r:id="rId2"/>
-    <sheet name="Interface Def and Reqs" sheetId="3" r:id="rId3"/>
+    <sheet name="Interface Definitions" sheetId="3" r:id="rId3"/>
     <sheet name="Requiremnts Unknowns" sheetId="2" r:id="rId4"/>
     <sheet name="OLD SoftwareRequirements" sheetId="1" r:id="rId5"/>
   </sheets>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="263">
   <si>
     <t>Name</t>
   </si>
@@ -303,15 +303,9 @@
     <t>SR-5-1</t>
   </si>
   <si>
-    <t>The service shall listen for and record all zones announced outside of this service</t>
-  </si>
-  <si>
     <t>The service shall subscribe to zone declaration messages</t>
   </si>
   <si>
-    <t>The service shall respond to received zone declaration messages by recording their full content</t>
-  </si>
-  <si>
     <t>The service shall subscribe to vehicle configuration messages</t>
   </si>
   <si>
@@ -435,9 +429,6 @@
     <t>The service shall pass received zone declarations to the ZoneAlert Computer</t>
   </si>
   <si>
-    <t>The ZoneAlertComputer shall store all zone information for each zone received</t>
-  </si>
-  <si>
     <t>ZoenAlertService</t>
   </si>
   <si>
@@ -636,9 +627,6 @@
     <t>The service shall log as an error any vehicle configurations or zones declared after it receives the event indicating that such declarations are complete</t>
   </si>
   <si>
-    <t>The service shall perform zone merging</t>
-  </si>
-  <si>
     <t>SR-6-1-1</t>
   </si>
   <si>
@@ -805,6 +793,42 @@
   </si>
   <si>
     <t>SR-7-4-6</t>
+  </si>
+  <si>
+    <t>The service shall perform zone merging using the standard defined zone merging semantcs</t>
+  </si>
+  <si>
+    <t>The service shall listen for and record all zones announced outside of this service as polygons in cartesian space equivalently to the geometry applied by RoutePlanner service</t>
+  </si>
+  <si>
+    <t>The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics</t>
+  </si>
+  <si>
+    <t>SR-4-3-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ZoneAlertComputer shall store all zone information for each zone as </t>
+  </si>
+  <si>
+    <t>Inptu Zone Requiremnts from service</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric applied in the RoutePlanning service.</t>
+  </si>
+  <si>
+    <t>no latitudes greater than 90 degrees or less than -90 degrees.</t>
+  </si>
+  <si>
+    <t>restricted lattitudes</t>
+  </si>
+  <si>
+    <t>altitudes are ignored</t>
+  </si>
+  <si>
+    <t>timespans ignored</t>
+  </si>
+  <si>
+    <t>relevant vehicles ignored</t>
   </si>
 </sst>
 </file>
@@ -1317,12 +1341,12 @@
         <v>72</v>
       </c>
       <c r="B1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B2" t="s">
         <v>73</v>
@@ -1330,10 +1354,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -1343,7 +1367,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34AC7C05-FC71-F749-BB41-F1A5141E29DB}">
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G99"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -1366,13 +1390,13 @@
         <v>85</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="52" thickTop="1" x14ac:dyDescent="0.2">
@@ -1383,16 +1407,16 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E2" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -1403,156 +1427,156 @@
         <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G5" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E6" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G6" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E7" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G7" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G8" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E9" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G9" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="F10" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G10" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -1560,33 +1584,33 @@
         <v>78</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F11" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>79</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>87</v>
+        <v>252</v>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
@@ -1594,19 +1618,19 @@
         <v>80</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E13" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G13" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1614,1181 +1638,1186 @@
         <v>81</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G14" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>89</v>
+        <v>253</v>
       </c>
       <c r="D15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E15" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G15" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D16" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E16" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F16" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G16" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>172</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="D17" t="s">
+        <v>123</v>
+      </c>
+      <c r="E17" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>175</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="D17" t="s">
-        <v>125</v>
-      </c>
-      <c r="E17" t="s">
-        <v>183</v>
-      </c>
       <c r="F17" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G17" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>254</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="16" t="s">
+      <c r="B19" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C19" t="s">
         <v>84</v>
       </c>
-      <c r="D18" t="s">
-        <v>124</v>
-      </c>
-      <c r="E18" t="s">
-        <v>155</v>
-      </c>
-      <c r="F18" t="s">
-        <v>124</v>
-      </c>
-      <c r="G18" t="s">
+      <c r="D19" t="s">
+        <v>122</v>
+      </c>
+      <c r="E19" t="s">
+        <v>152</v>
+      </c>
+      <c r="F19" t="s">
+        <v>122</v>
+      </c>
+      <c r="G19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D20" t="s">
+        <v>122</v>
+      </c>
+      <c r="E20" t="s">
+        <v>152</v>
+      </c>
+      <c r="F20" t="s">
+        <v>122</v>
+      </c>
+      <c r="G20" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="16" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="D19" t="s">
-        <v>124</v>
-      </c>
-      <c r="E19" t="s">
-        <v>155</v>
-      </c>
-      <c r="F19" t="s">
-        <v>124</v>
-      </c>
-      <c r="G19" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>91</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>184</v>
-      </c>
-      <c r="E20" t="s">
-        <v>155</v>
-      </c>
-      <c r="F20" t="s">
-        <v>124</v>
-      </c>
-      <c r="G20" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="E21" t="s">
+        <v>152</v>
+      </c>
+      <c r="F21" t="s">
+        <v>122</v>
+      </c>
+      <c r="G21" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>182</v>
+      </c>
+      <c r="B22" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="B21" s="16" t="s">
-        <v>188</v>
-      </c>
-      <c r="D21" t="s">
-        <v>132</v>
-      </c>
-      <c r="E21" t="s">
-        <v>155</v>
-      </c>
-      <c r="F21" t="s">
-        <v>124</v>
-      </c>
-      <c r="G21" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>186</v>
-      </c>
-      <c r="B22" s="16" t="s">
-        <v>190</v>
-      </c>
       <c r="D22" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="E22" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F22" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G22" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>133</v>
+        <v>187</v>
       </c>
       <c r="D23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E23" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="F23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G23" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>92</v>
+        <v>188</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>198</v>
+        <v>130</v>
+      </c>
+      <c r="D24" t="s">
+        <v>123</v>
       </c>
       <c r="E24" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="F24" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>123</v>
+      </c>
+      <c r="G24" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="D25" t="s">
-        <v>124</v>
+        <v>251</v>
       </c>
       <c r="E25" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F25" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>199</v>
+        <v>93</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>94</v>
+        <v>192</v>
       </c>
       <c r="D26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E26" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F26" t="s">
-        <v>124</v>
-      </c>
-      <c r="G26" t="s">
-        <v>159</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E27" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F27" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G27" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>202</v>
+        <v>95</v>
+      </c>
+      <c r="D28" t="s">
+        <v>122</v>
       </c>
       <c r="E28" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G28" t="s">
-        <v>203</v>
+        <v>178</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>96</v>
+        <v>197</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="E29" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="F29" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G29" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>205</v>
-      </c>
-      <c r="D30" t="s">
-        <v>124</v>
+        <v>200</v>
       </c>
       <c r="E30" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F30" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G30" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>192</v>
+        <v>96</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="D31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E31" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F31" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G31" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>189</v>
+      </c>
+      <c r="B32" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D32" t="s">
+        <v>122</v>
+      </c>
+      <c r="E32" t="s">
+        <v>180</v>
+      </c>
+      <c r="F32" t="s">
+        <v>123</v>
+      </c>
+      <c r="G32" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>190</v>
+      </c>
+      <c r="B33" s="16" t="s">
+        <v>147</v>
+      </c>
+      <c r="E33" t="s">
+        <v>180</v>
+      </c>
+      <c r="F33" t="s">
+        <v>123</v>
+      </c>
+      <c r="G33" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" ht="85" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>193</v>
-      </c>
-      <c r="B32" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="E32" t="s">
-        <v>183</v>
-      </c>
-      <c r="F32" t="s">
-        <v>125</v>
-      </c>
-      <c r="G32" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>207</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="E33" t="s">
-        <v>183</v>
-      </c>
-      <c r="F33" t="s">
-        <v>125</v>
-      </c>
-      <c r="G33" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>208</v>
-      </c>
       <c r="B34" s="16" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F34" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G34" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E35" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F35" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G35" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="D36" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="E36" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F36" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G36" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>99</v>
+        <v>151</v>
       </c>
       <c r="D37" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F37" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G37" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E38" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F38" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G38" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>211</v>
+        <v>193</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E39" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="F39" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="G39" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>213</v>
+        <v>103</v>
+      </c>
+      <c r="D40" t="s">
+        <v>122</v>
       </c>
       <c r="E40" t="s">
-        <v>183</v>
+        <v>152</v>
       </c>
       <c r="F40" t="s">
-        <v>125</v>
-      </c>
-      <c r="G40" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="D41" t="s">
-        <v>125</v>
+        <v>209</v>
       </c>
       <c r="E41" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F41" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G41" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>220</v>
+        <v>132</v>
+      </c>
+      <c r="D42" t="s">
+        <v>123</v>
       </c>
       <c r="E42" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F42" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G42" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="E43" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F43" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G43" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="E44" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F44" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G44" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>216</v>
-      </c>
-      <c r="D45" t="s">
-        <v>124</v>
+        <v>218</v>
       </c>
       <c r="E45" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="F45" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G45" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>106</v>
+        <v>212</v>
       </c>
       <c r="D46" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="E46" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F46" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G46" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D47" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E47" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F47" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G47" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B48" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="D48" t="s">
+        <v>133</v>
+      </c>
+      <c r="E48" t="s">
+        <v>152</v>
+      </c>
+      <c r="F48" t="s">
+        <v>122</v>
+      </c>
+      <c r="G48" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>215</v>
+      </c>
+      <c r="B49" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="D49" t="s">
+        <v>133</v>
+      </c>
+      <c r="E49" t="s">
+        <v>152</v>
+      </c>
+      <c r="F49" t="s">
+        <v>122</v>
+      </c>
+      <c r="G49" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>99</v>
+      </c>
+      <c r="B50" s="16" t="s">
+        <v>240</v>
+      </c>
+      <c r="D50" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50" t="s">
+        <v>152</v>
+      </c>
+      <c r="F50" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>91</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="E51" t="s">
+        <v>152</v>
+      </c>
+      <c r="F51" t="s">
+        <v>122</v>
+      </c>
+      <c r="G51" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>100</v>
+      </c>
+      <c r="B52" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D52" t="s">
+        <v>122</v>
+      </c>
+      <c r="E52" t="s">
+        <v>152</v>
+      </c>
+      <c r="F52" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>224</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="D53" t="s">
+        <v>122</v>
+      </c>
+      <c r="E53" t="s">
+        <v>152</v>
+      </c>
+      <c r="F53" t="s">
+        <v>122</v>
+      </c>
+      <c r="G53" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>225</v>
+      </c>
+      <c r="B54" s="16" t="s">
+        <v>134</v>
+      </c>
+      <c r="D54" t="s">
+        <v>122</v>
+      </c>
+      <c r="E54" t="s">
+        <v>152</v>
+      </c>
+      <c r="F54" t="s">
+        <v>122</v>
+      </c>
+      <c r="G54" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>227</v>
+      </c>
+      <c r="B55" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="D55" t="s">
+        <v>123</v>
+      </c>
+      <c r="E55" t="s">
+        <v>180</v>
+      </c>
+      <c r="F55" t="s">
+        <v>123</v>
+      </c>
+      <c r="G55" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>229</v>
+      </c>
+      <c r="B56" s="16" t="s">
         <v>136</v>
       </c>
-      <c r="E48" t="s">
-        <v>155</v>
-      </c>
-      <c r="F48" t="s">
-        <v>124</v>
-      </c>
-      <c r="G48" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" ht="85" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>101</v>
-      </c>
-      <c r="B49" s="16" t="s">
-        <v>244</v>
-      </c>
-      <c r="D49" t="s">
-        <v>124</v>
-      </c>
-      <c r="E49" t="s">
-        <v>155</v>
-      </c>
-      <c r="F49" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>93</v>
-      </c>
-      <c r="B50" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="E50" t="s">
-        <v>155</v>
-      </c>
-      <c r="F50" t="s">
-        <v>124</v>
-      </c>
-      <c r="G50" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
-        <v>102</v>
-      </c>
-      <c r="B51" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="D51" t="s">
-        <v>124</v>
-      </c>
-      <c r="E51" t="s">
-        <v>155</v>
-      </c>
-      <c r="F51" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="D56" t="s">
+        <v>123</v>
+      </c>
+      <c r="E56" t="s">
+        <v>180</v>
+      </c>
+      <c r="F56" t="s">
+        <v>123</v>
+      </c>
+      <c r="G56" t="s">
         <v>228</v>
-      </c>
-      <c r="B52" s="16" t="s">
-        <v>227</v>
-      </c>
-      <c r="D52" t="s">
-        <v>124</v>
-      </c>
-      <c r="E52" t="s">
-        <v>155</v>
-      </c>
-      <c r="F52" t="s">
-        <v>124</v>
-      </c>
-      <c r="G52" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>229</v>
-      </c>
-      <c r="B53" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="D53" t="s">
-        <v>124</v>
-      </c>
-      <c r="E53" t="s">
-        <v>155</v>
-      </c>
-      <c r="F53" t="s">
-        <v>124</v>
-      </c>
-      <c r="G53" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>231</v>
-      </c>
-      <c r="B54" s="16" t="s">
-        <v>138</v>
-      </c>
-      <c r="D54" t="s">
-        <v>125</v>
-      </c>
-      <c r="E54" t="s">
-        <v>183</v>
-      </c>
-      <c r="F54" t="s">
-        <v>125</v>
-      </c>
-      <c r="G54" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>233</v>
-      </c>
-      <c r="B55" s="16" t="s">
-        <v>139</v>
-      </c>
-      <c r="D55" t="s">
-        <v>125</v>
-      </c>
-      <c r="E55" t="s">
-        <v>183</v>
-      </c>
-      <c r="F55" t="s">
-        <v>125</v>
-      </c>
-      <c r="G55" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="85" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>234</v>
-      </c>
-      <c r="B56" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="D56" t="s">
-        <v>125</v>
-      </c>
-      <c r="E56" t="s">
-        <v>183</v>
-      </c>
-      <c r="F56" t="s">
-        <v>125</v>
-      </c>
-      <c r="G56" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>236</v>
+        <v>138</v>
+      </c>
+      <c r="D57" t="s">
+        <v>123</v>
       </c>
       <c r="E57" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F57" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G57" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>231</v>
+      </c>
+      <c r="B58" s="16" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A58" s="14" t="s">
-        <v>237</v>
-      </c>
-      <c r="B58" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="D58" t="s">
-        <v>125</v>
-      </c>
       <c r="E58" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F58" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G58" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="D59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E59" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G59" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
         <v>239</v>
       </c>
       <c r="B60" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D60" t="s">
+        <v>123</v>
+      </c>
+      <c r="E60" t="s">
+        <v>180</v>
+      </c>
+      <c r="F60" t="s">
+        <v>123</v>
+      </c>
+      <c r="G60" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+      <c r="A61" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="B61" s="16" t="s">
+        <v>234</v>
+      </c>
+      <c r="D61" t="s">
+        <v>123</v>
+      </c>
+      <c r="E61" t="s">
+        <v>180</v>
+      </c>
+      <c r="F61" t="s">
+        <v>123</v>
+      </c>
+      <c r="G61" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A62" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B62" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="E62" t="s">
+        <v>180</v>
+      </c>
+      <c r="F62" t="s">
+        <v>123</v>
+      </c>
+      <c r="G62" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>237</v>
+      </c>
+      <c r="B63" s="16" t="s">
         <v>238</v>
       </c>
-      <c r="D60" t="s">
-        <v>125</v>
-      </c>
-      <c r="E60" t="s">
-        <v>183</v>
-      </c>
-      <c r="F60" t="s">
-        <v>125</v>
-      </c>
-      <c r="G60" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A61" s="14" t="s">
-        <v>240</v>
-      </c>
-      <c r="B61" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E61" t="s">
-        <v>183</v>
-      </c>
-      <c r="F61" t="s">
-        <v>125</v>
-      </c>
-      <c r="G61" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" ht="102" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>241</v>
-      </c>
-      <c r="B62" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="E62" t="s">
-        <v>183</v>
-      </c>
-      <c r="F62" t="s">
-        <v>125</v>
-      </c>
-      <c r="G62" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>103</v>
-      </c>
-      <c r="B63" s="16" t="s">
-        <v>111</v>
-      </c>
       <c r="E63" t="s">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="F63" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="G63" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>245</v>
+        <v>101</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E64" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F64" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G64" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E65" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F65" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G65" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E66" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F66" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G66" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="B67" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="E67" t="s">
+        <v>152</v>
+      </c>
+      <c r="F67" t="s">
+        <v>122</v>
+      </c>
+      <c r="G67" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>244</v>
+      </c>
+      <c r="B68" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="E68" t="s">
+        <v>152</v>
+      </c>
+      <c r="F68" t="s">
+        <v>122</v>
+      </c>
+      <c r="G68" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>245</v>
+      </c>
+      <c r="B69" s="16" t="s">
+        <v>114</v>
+      </c>
+      <c r="E69" t="s">
+        <v>152</v>
+      </c>
+      <c r="F69" t="s">
+        <v>122</v>
+      </c>
+      <c r="G69" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>246</v>
+      </c>
+      <c r="B70" s="16" t="s">
+        <v>116</v>
+      </c>
+      <c r="E70" t="s">
+        <v>152</v>
+      </c>
+      <c r="F70" t="s">
+        <v>122</v>
+      </c>
+      <c r="G70" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>247</v>
+      </c>
+      <c r="B71" s="16" t="s">
         <v>115</v>
       </c>
-      <c r="E67" t="s">
-        <v>155</v>
-      </c>
-      <c r="F67" t="s">
-        <v>124</v>
-      </c>
-      <c r="G67" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>249</v>
-      </c>
-      <c r="B68" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="E68" t="s">
-        <v>155</v>
-      </c>
-      <c r="F68" t="s">
-        <v>124</v>
-      </c>
-      <c r="G68" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>250</v>
-      </c>
-      <c r="B69" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="E69" t="s">
-        <v>155</v>
-      </c>
-      <c r="F69" t="s">
-        <v>124</v>
-      </c>
-      <c r="G69" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>251</v>
-      </c>
-      <c r="B70" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="E70" t="s">
-        <v>155</v>
-      </c>
-      <c r="F70" t="s">
-        <v>124</v>
-      </c>
-      <c r="G70" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>252</v>
-      </c>
-      <c r="B71" s="16" t="s">
-        <v>120</v>
-      </c>
       <c r="E71" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F71" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G71" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E72" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F72" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G72" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E73" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F73" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G73" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>104</v>
+        <v>250</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E74" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F74" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G74" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="D75" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E75" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F75" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G75" t="s">
-        <v>181</v>
+        <v>226</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>176</v>
+        <v>107</v>
       </c>
       <c r="B76" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="D76" t="s">
+        <v>122</v>
+      </c>
+      <c r="E76" t="s">
+        <v>152</v>
+      </c>
+      <c r="F76" t="s">
+        <v>122</v>
+      </c>
+      <c r="G76" t="s">
         <v>178</v>
-      </c>
-      <c r="E76" t="s">
-        <v>183</v>
-      </c>
-      <c r="F76" t="s">
-        <v>125</v>
-      </c>
-      <c r="G76" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E77" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F77" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G77" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B78" s="16"/>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>174</v>
+      </c>
+      <c r="B78" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="E78" t="s">
+        <v>180</v>
+      </c>
+      <c r="F78" t="s">
+        <v>123</v>
+      </c>
+      <c r="G78" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B79" s="16"/>
@@ -2800,7 +2829,7 @@
       <c r="B81" s="16"/>
     </row>
     <row r="82" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B82" s="18"/>
+      <c r="B82" s="16"/>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B83" s="18"/>
@@ -2809,10 +2838,10 @@
       <c r="B84" s="18"/>
     </row>
     <row r="85" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B85" s="16"/>
+      <c r="B85" s="18"/>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B86" s="18"/>
+      <c r="B86" s="16"/>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B87" s="18"/>
@@ -2825,13 +2854,13 @@
     </row>
     <row r="90" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B90" s="18"/>
-      <c r="C90" s="13"/>
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B91" s="16"/>
+      <c r="B91" s="18"/>
+      <c r="C91" s="13"/>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B92" s="18"/>
+      <c r="B92" s="16"/>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B93" s="18"/>
@@ -2849,7 +2878,10 @@
       <c r="B97" s="18"/>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B98" s="16"/>
+      <c r="B98" s="18"/>
+    </row>
+    <row r="99" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B99" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2859,9 +2891,43 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3702B00E-AAB7-7F4B-9F1C-57A3CF73FDCB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Updated issues and requirements based on a few bugs found while working on compositional testing.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D260B86-EAE2-F648-BE4C-5D50B132DA77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAC9518-1E87-A24C-A9BA-56E9E0FB7070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="2" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="262">
   <si>
     <t>Name</t>
   </si>
@@ -327,18 +327,9 @@
     <t>SR-6-2</t>
   </si>
   <si>
-    <t>The service shall respond to the first received event indicating that OpenUxAS environment and vehicle declarations are complete by performing zone merging</t>
-  </si>
-  <si>
     <t>SR-6-2-1</t>
   </si>
   <si>
-    <t>The service assign a unique id to each resulting merged zone</t>
-  </si>
-  <si>
-    <t>The service shall store all created merged zones</t>
-  </si>
-  <si>
     <t>SR-7</t>
   </si>
   <si>
@@ -432,15 +423,6 @@
     <t>ZoenAlertService</t>
   </si>
   <si>
-    <t>The ZoneAlerComputer shall store zone declarations mapped from ID to vehicle cofig declaration</t>
-  </si>
-  <si>
-    <t>Authoritative Zone Merging Module</t>
-  </si>
-  <si>
-    <t>The Zone Alert Computer mergeZones function shall return the sets of created merged zones, both keep-in and keep-out, providing a merged zone's id and its full geometry for each and every such created merged zone</t>
-  </si>
-  <si>
     <t>ZoneAlertService, CMASI</t>
   </si>
   <si>
@@ -465,9 +447,6 @@
     <t>The zone alert computer shall compute the position and time of a detected existing zone violation between a vehicle's stated position and a merged zone as the stated vehicle position and time of the vehicle state report.</t>
   </si>
   <si>
-    <t>The service shal utilize the same semantics for zone geometry as route planning service</t>
-  </si>
-  <si>
     <t>OpenUxAS shall be aware of existing zone violations by vehicles to usefully avoiid/recover/accept imminent and existing zone violations.</t>
   </si>
   <si>
@@ -483,21 +462,6 @@
     <t>The installed ZoneAlertComputer shall determine whether a given time window is acceptable to it to be able to effectivel compute imminent zone alerts</t>
   </si>
   <si>
-    <t xml:space="preserve">The Authoritative Zone Merging Model shall merge all zones such that all zones of the same type (keep-in or keep-out) are merged into a single zone with each and every zone of the same type with which they overlap or touch in the horizontal plane. </t>
-  </si>
-  <si>
-    <t>The Authoritative Zone Merging Model shall merge all zones such that all zones conserve their initial encompassed area in the horizontal plane.</t>
-  </si>
-  <si>
-    <t>The Authoritative Zone Merging Model shall merge zones shall allow internal holes that are created in the merging of a zone to be ignored, including that area in the resulting merged zones in the horizontal plane</t>
-  </si>
-  <si>
-    <t>The Authoritative Zone Merging Model shall not create geometry in the vertical plane, with the assumption that all altitudes are included in the merged zone semantics.</t>
-  </si>
-  <si>
-    <t>The Authoritative Zone Merging Model shall merge overlapping zones in the x-y plane with the same semantics of the prefered OpenUxAS Route Planning service</t>
-  </si>
-  <si>
     <t>ZoneAlertService.h</t>
   </si>
   <si>
@@ -612,15 +576,6 @@
     <t>SR-6-2-2</t>
   </si>
   <si>
-    <t>SR-6-2-3</t>
-  </si>
-  <si>
-    <t>SR-6-2-4</t>
-  </si>
-  <si>
-    <t>The service shall perform zone merging immediately after receiving an OpenUxAS message indicating that the system is done declaring vehicles and zones.</t>
-  </si>
-  <si>
     <t>SR-6-3</t>
   </si>
   <si>
@@ -633,87 +588,27 @@
     <t>SR-6-1-2</t>
   </si>
   <si>
-    <t>SR-6-1-3</t>
-  </si>
-  <si>
-    <t>The service shall command the Zone Alert Computer to perform the zone merging</t>
-  </si>
-  <si>
     <t>mergeZones</t>
   </si>
   <si>
-    <t>The Zone Alert Computer shall merging zones using the defined zone merging semantics</t>
-  </si>
-  <si>
-    <t>The service shall merge all and only keep in zones into overlaping merged keep-in zones using the defined merging semantics</t>
-  </si>
-  <si>
-    <t>The service shall merge all and only keep out zones into overlaping merged keep-out zones using the defined merging semantics</t>
-  </si>
-  <si>
-    <t>SR-6-2-3-1</t>
-  </si>
-  <si>
-    <t>SR-6-2-3-2</t>
-  </si>
-  <si>
-    <t>SR-6-2-3-3</t>
-  </si>
-  <si>
-    <t>SR-6-2-3-4</t>
-  </si>
-  <si>
     <t>SR-6-4</t>
   </si>
   <si>
     <t>SR-6-4-1</t>
   </si>
   <si>
-    <t>The Zone Alert Computer shall return the set of all and only  merged zones from its zone merging computation</t>
-  </si>
-  <si>
-    <t>SR-6-4-2</t>
-  </si>
-  <si>
-    <t>SR-6-4-3</t>
-  </si>
-  <si>
     <t>The Zone Alert Service shall take the set of returned merged zones and announce each and every one as a Merged Zone Declaration to OpenUxAS as OpenUxAS event/messages</t>
   </si>
   <si>
-    <t>SR-6-4-3-1</t>
-  </si>
-  <si>
-    <t>SR-6-4-3-2</t>
-  </si>
-  <si>
-    <t>SR-6-4-3-3</t>
-  </si>
-  <si>
-    <t>Each merged zone declaration shall state the assigned ID of the merged zone</t>
-  </si>
-  <si>
     <t>Each merged zone declaration shall state the geometry of the merged zone polyhedron</t>
   </si>
   <si>
     <t>Each merged zone declaration shall state whether the merged zone is keep-out or keep-in</t>
   </si>
   <si>
-    <t>SR-6-4-2-1</t>
-  </si>
-  <si>
-    <t>SR-6-4-2-2</t>
-  </si>
-  <si>
-    <t>SR-6-4-2-3</t>
-  </si>
-  <si>
     <t>The zone alert service shall subscribe to vehicle state messages when the service initiates</t>
   </si>
   <si>
-    <t>The zone alert service shall respond to a received vehicle state by computing whether a violation exists between the received vehicle state and each merged zone</t>
-  </si>
-  <si>
     <t>SR-7-3</t>
   </si>
   <si>
@@ -795,27 +690,12 @@
     <t>SR-7-4-6</t>
   </si>
   <si>
-    <t>The service shall perform zone merging using the standard defined zone merging semantcs</t>
-  </si>
-  <si>
     <t>The service shall listen for and record all zones announced outside of this service as polygons in cartesian space equivalently to the geometry applied by RoutePlanner service</t>
   </si>
   <si>
-    <t>The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics</t>
-  </si>
-  <si>
-    <t>SR-4-3-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The ZoneAlertComputer shall store all zone information for each zone as </t>
-  </si>
-  <si>
     <t>Inptu Zone Requiremnts from service</t>
   </si>
   <si>
-    <t>The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric applied in the RoutePlanning service.</t>
-  </si>
-  <si>
     <t>no latitudes greater than 90 degrees or less than -90 degrees.</t>
   </si>
   <si>
@@ -829,6 +709,123 @@
   </si>
   <si>
     <t>relevant vehicles ignored</t>
+  </si>
+  <si>
+    <t>SR-4-3-2-1</t>
+  </si>
+  <si>
+    <t>The service shal utilize the same semantics for zone geometry as route planning service except that resulting degenerate zones are allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics when it uses the bFIndPointsForAbstractGeometry method. </t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric applied in the RoutePlannerVisbilityService when it calls bFindPointsForAbstractGeometry method</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall store all declared abstract geometries by calling the same bFindPointsForAbstractGeometry function as used by RoutePLannerVisibilityService.</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall perform zone merging with RoutePlannerVisibilityService by constructing an empty VisbilityGraph and processing zone polygons as is performed by the RoutePlannerVisibilityService.</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall return that no zones are created for zone alerting if the errFinalizePolygons function returns an error code.</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall follow construction of its empty VisibilityGraph by processing zone polygons as is performed by the RoutePlannerVisibilityService.</t>
+  </si>
+  <si>
+    <t>SR-6-2-2-1</t>
+  </si>
+  <si>
+    <t>SR-6-2-2-2</t>
+  </si>
+  <si>
+    <t>SR-6-2-2-3</t>
+  </si>
+  <si>
+    <t>SR-6-2-2-4</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall iteratively attempt to add each zone polygon to the VisibilityGraph using the errAddPolygon function, just as the RoutePlannerVisibilityService does.</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall respond to an error return value for any call of errAddPolygon by ceasing to attempt to add declared zone polgons to the visbility graph, and instead returning that no zones have been constructed for zone alerting.</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall follow up complete iteration over all zones calling errAddPolygon with no error condition returned on any call by calling errFInalizePolygons on the visibility graph</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall return the set of all and only zone polygon boundaries defined in the VisibilitGraph if errFinalizePolygons is called and returns that no error has occurred.</t>
+  </si>
+  <si>
+    <t>SR-6-2-2-5</t>
+  </si>
+  <si>
+    <t>The Zone Alert COmputer assign a unique id to each resulting merged zone created as output of the VisibilityGraph</t>
+  </si>
+  <si>
+    <t>When all zones are finished being declared by OpenUxAS, rhe service shall perform zone checking, explansion, and merging using the standard defined zone processing semantcs of the RoutePlannerVisbilityService when an Operating Region is declared</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The zone service shall expand, merge, and check all zones using the same semantics </t>
+  </si>
+  <si>
+    <t>The service shall command the Zone Alert Computer to perform the zone checking, expansion, and merging using the same semantics of the RoutePlannerVisibilityService when an Operating Region is declared</t>
+  </si>
+  <si>
+    <t>Having processed, merged, and checked zones by command of the service, the ZoneAlertComputer will then organize , store for later use, and return the set of resulting zones to the Zone Alert Service.</t>
+  </si>
+  <si>
+    <t>SR-6-3-1</t>
+  </si>
+  <si>
+    <t>SR-6-3-2</t>
+  </si>
+  <si>
+    <t>SR-6-3-3</t>
+  </si>
+  <si>
+    <t>The ZoneAletComputer shall return the set of all and only resulting processed zones to the Zone Alert Service.</t>
+  </si>
+  <si>
+    <t>SR-6-3-3-1</t>
+  </si>
+  <si>
+    <t>SR-6-4-1-1</t>
+  </si>
+  <si>
+    <t>SR-6-4-1-2</t>
+  </si>
+  <si>
+    <t>SR-6-4-1-3</t>
+  </si>
+  <si>
+    <t>Each merged zone returned shall state the assigned ID of the merged zone</t>
+  </si>
+  <si>
+    <t>When called to do so, The Zone Alert Computer shall process, check, and merge zones using the defined zone checking, expansion and merging semantics of the RoutePlannerVisibilityService when an OperatingRegions is declared</t>
+  </si>
+  <si>
+    <t>The ZoneAlertCOmputer shall store all created merged zones for later Zone Alerting</t>
+  </si>
+  <si>
+    <t>SR-6-3-3-2</t>
+  </si>
+  <si>
+    <t>SR-6-3-3-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The service shall respond to the first received event indicating that OpenUxAS environment and vehicle declarations are complete by performing zone expanding, merging, and checking. </t>
+  </si>
+  <si>
+    <t>SR-6-1-2-1</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall store vehicle declarations mapped from ID to vehicle config declaration</t>
+  </si>
+  <si>
+    <t>The zone alert service shall respond to a received vehicle state by correctly determining whether a violation exists between the received vehicle state and each merged zone</t>
   </si>
 </sst>
 </file>
@@ -1341,12 +1338,12 @@
         <v>72</v>
       </c>
       <c r="B1" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B2" t="s">
         <v>73</v>
@@ -1354,10 +1351,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>141</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -1390,13 +1387,13 @@
         <v>85</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="52" thickTop="1" x14ac:dyDescent="0.2">
@@ -1407,16 +1404,16 @@
         <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E2" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G2" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -1427,156 +1424,156 @@
         <v>74</v>
       </c>
       <c r="D3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E3" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E4" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G5" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E6" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G6" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E7" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F7" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G7" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>164</v>
+        <v>152</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
       <c r="D8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E8" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G8" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F9" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G9" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>154</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E10" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="F10" t="s">
-        <v>168</v>
+        <v>156</v>
       </c>
       <c r="G10" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -1584,16 +1581,16 @@
         <v>78</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="D11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E11" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.2">
@@ -1601,16 +1598,16 @@
         <v>79</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>252</v>
+        <v>216</v>
       </c>
       <c r="D12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E12" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
@@ -1621,16 +1618,16 @@
         <v>87</v>
       </c>
       <c r="D13" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E13" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F13" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G13" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1638,87 +1635,99 @@
         <v>81</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>169</v>
+        <v>157</v>
       </c>
       <c r="D14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E14" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F14" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G14" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>253</v>
+        <v>225</v>
       </c>
       <c r="D15" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E15" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F15" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G15" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E16" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F16" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G16" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>172</v>
+        <v>160</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>257</v>
+        <v>226</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E17" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F17" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G17" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>254</v>
+        <v>223</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>255</v>
+        <v>227</v>
+      </c>
+      <c r="D18" t="s">
+        <v>120</v>
+      </c>
+      <c r="E18" t="s">
+        <v>168</v>
+      </c>
+      <c r="F18" t="s">
+        <v>120</v>
+      </c>
+      <c r="G18" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1732,16 +1741,16 @@
         <v>84</v>
       </c>
       <c r="D19" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F19" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G19" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
@@ -1752,16 +1761,16 @@
         <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G20" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1769,76 +1778,76 @@
         <v>89</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="E21" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F21" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G21" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D22" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E22" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F22" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G22" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="D23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E23" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F23" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G23" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>130</v>
+        <v>260</v>
       </c>
       <c r="D24" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E24" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F24" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G24" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -1846,474 +1855,477 @@
         <v>90</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="E25" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F25" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>93</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>192</v>
+        <v>241</v>
       </c>
       <c r="D26" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E26" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F26" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="B27" s="16" t="s">
         <v>92</v>
       </c>
       <c r="D27" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E27" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F27" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G27" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>95</v>
+        <v>258</v>
       </c>
       <c r="D28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E28" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G28" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>197</v>
+        <v>259</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>198</v>
+        <v>243</v>
       </c>
       <c r="E29" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F29" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G29" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>94</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>200</v>
+        <v>254</v>
       </c>
       <c r="E30" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F30" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G30" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>201</v>
+        <v>228</v>
       </c>
       <c r="D31" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E31" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F31" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G31" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>202</v>
-      </c>
-      <c r="D32" t="s">
-        <v>122</v>
-      </c>
-      <c r="E32" t="s">
-        <v>180</v>
-      </c>
-      <c r="F32" t="s">
-        <v>123</v>
-      </c>
-      <c r="G32" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>190</v>
+        <v>231</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>147</v>
+        <v>235</v>
+      </c>
+      <c r="D33" t="s">
+        <v>119</v>
       </c>
       <c r="E33" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F33" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G33" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>148</v>
+        <v>236</v>
       </c>
       <c r="E34" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F34" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G34" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>149</v>
+        <v>237</v>
       </c>
       <c r="E35" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F35" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G35" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>150</v>
+        <v>229</v>
       </c>
       <c r="E36" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F36" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G36" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>206</v>
+        <v>239</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>151</v>
-      </c>
-      <c r="D37" t="s">
-        <v>131</v>
+        <v>238</v>
       </c>
       <c r="E37" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F37" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G37" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>97</v>
+        <v>244</v>
       </c>
       <c r="D38" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E38" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F38" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G38" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>193</v>
+        <v>245</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>98</v>
+        <v>240</v>
       </c>
       <c r="D39" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E39" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F39" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G39" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>207</v>
+        <v>246</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>103</v>
+        <v>255</v>
       </c>
       <c r="D40" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E40" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="F40" t="s">
-        <v>122</v>
+        <v>120</v>
+      </c>
+      <c r="G40" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>208</v>
+        <v>247</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>209</v>
+        <v>248</v>
+      </c>
+      <c r="D41" t="s">
+        <v>120</v>
       </c>
       <c r="E41" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F41" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G41" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>210</v>
+        <v>249</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>132</v>
+        <v>253</v>
       </c>
       <c r="D42" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E42" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F42" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G42" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>216</v>
+        <v>186</v>
+      </c>
+      <c r="D43" t="s">
+        <v>120</v>
       </c>
       <c r="E43" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F43" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G43" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>220</v>
+        <v>257</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>217</v>
+        <v>187</v>
+      </c>
+      <c r="D44" t="s">
+        <v>120</v>
       </c>
       <c r="E44" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F44" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G44" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>221</v>
+        <v>183</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>218</v>
+        <v>100</v>
+      </c>
+      <c r="D45" t="s">
+        <v>119</v>
       </c>
       <c r="E45" t="s">
-        <v>180</v>
+        <v>140</v>
       </c>
       <c r="F45" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G45" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>211</v>
+        <v>184</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>212</v>
+        <v>185</v>
       </c>
       <c r="D46" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E46" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F46" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G46" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D47" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E47" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F47" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G47" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D48" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E48" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F48" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G48" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D49" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E49" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F49" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G49" t="s">
-        <v>199</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="D50" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E50" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F50" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
@@ -2321,502 +2333,502 @@
         <v>91</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="E51" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F51" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G51" t="s">
-        <v>156</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D52" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E52" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F52" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>224</v>
+        <v>189</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>223</v>
+        <v>261</v>
       </c>
       <c r="D53" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E53" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F53" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G53" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>225</v>
+        <v>190</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D54" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E54" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F54" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G54" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>227</v>
+        <v>192</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D55" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E55" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F55" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G55" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D56" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E56" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F56" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G56" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D57" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E57" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F57" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G57" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>231</v>
+        <v>196</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>232</v>
+        <v>197</v>
       </c>
       <c r="E58" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F58" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G58" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A59" s="14" t="s">
-        <v>233</v>
+        <v>198</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D59" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E59" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F59" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G59" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>239</v>
+        <v>204</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D60" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E60" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F60" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G60" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="153" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>234</v>
+        <v>199</v>
       </c>
       <c r="D61" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E61" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F61" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G61" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>236</v>
+        <v>201</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E62" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F62" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G62" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>237</v>
+        <v>202</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>238</v>
+        <v>203</v>
       </c>
       <c r="E63" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F63" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G63" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="E64" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F64" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G64" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>241</v>
+        <v>206</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E65" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F65" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G65" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>242</v>
+        <v>207</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E66" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F66" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G66" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>243</v>
+        <v>208</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E67" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F67" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G67" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>244</v>
+        <v>209</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E68" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F68" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G68" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>245</v>
+        <v>210</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E69" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F69" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G69" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>246</v>
+        <v>211</v>
       </c>
       <c r="B70" s="16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E70" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F70" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G70" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>247</v>
+        <v>212</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E71" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F71" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G71" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>248</v>
+        <v>213</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E72" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F72" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G72" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>249</v>
+        <v>214</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="E73" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F73" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G73" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E74" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F74" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G74" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E75" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F75" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G75" t="s">
-        <v>226</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B76" s="16" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="D76" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="E76" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="F76" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="G76" t="s">
-        <v>178</v>
+        <v>166</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="E77" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F77" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G77" t="s">
-        <v>199</v>
+        <v>182</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="E78" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
       <c r="F78" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="G78" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.2">
@@ -2896,35 +2908,35 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>256</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="B2" t="s">
-        <v>258</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>259</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>260</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>261</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>262</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial HL-1-2 argument with associated issues.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CBB143-000B-EB4F-8B60-A4B149D041C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878297AD-C290-6A44-A429-4B3A8ECF2DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="270">
   <si>
     <t>Name</t>
   </si>
@@ -714,12 +714,6 @@
     <t>SR-4-3-2-1</t>
   </si>
   <si>
-    <t>The service shal utilize the same semantics for zone geometry as route planning service except that resulting degenerate zones are allowed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics when it uses the bFIndPointsForAbstractGeometry method. </t>
-  </si>
-  <si>
     <t>The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric applied in the RoutePlannerVisbilityService when it calls bFindPointsForAbstractGeometry method</t>
   </si>
   <si>
@@ -826,6 +820,36 @@
   </si>
   <si>
     <t>The zone alert service shall respond to a received vehicle state by correctly determining whether a violation exists between the received vehicle state and each merged zone</t>
+  </si>
+  <si>
+    <t>The service shal utilize the same semantics for zone geometry as RoutePlannerVisibilityService</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics </t>
+  </si>
+  <si>
+    <t>HL-1-3</t>
+  </si>
+  <si>
+    <t>The service shall compute zone violations against zone semantics both correctly and accurately</t>
+  </si>
+  <si>
+    <t>HL-1-3-1</t>
+  </si>
+  <si>
+    <t>HL-1-3-2</t>
+  </si>
+  <si>
+    <t>HL-1-3-3</t>
+  </si>
+  <si>
+    <t>Zone geometry applied is isufficiently correct and accurate</t>
+  </si>
+  <si>
+    <t>Computation of existing zone violations is correct and accurate with respect to a vehicle state event</t>
+  </si>
+  <si>
+    <t>Computation of imminent zone violations is correct and accurate with respect to vehicle state events and linear immediate trajectory</t>
   </si>
 </sst>
 </file>
@@ -1327,7 +1351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FDF8AA6-5D75-9940-86F4-A0A21993176A}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="45.5" customWidth="1"/>
@@ -1354,7 +1378,39 @@
         <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>224</v>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>265</v>
+      </c>
+      <c r="B6" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>266</v>
+      </c>
+      <c r="B7" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -1650,12 +1706,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>158</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>225</v>
+        <v>261</v>
       </c>
       <c r="D15" t="s">
         <v>119</v>
@@ -1695,7 +1751,7 @@
         <v>160</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D17" t="s">
         <v>120</v>
@@ -1715,7 +1771,7 @@
         <v>223</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D18" t="s">
         <v>120</v>
@@ -1835,7 +1891,7 @@
         <v>176</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D24" t="s">
         <v>120</v>
@@ -1855,7 +1911,7 @@
         <v>90</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="E25" t="s">
         <v>140</v>
@@ -1869,7 +1925,7 @@
         <v>93</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D26" t="s">
         <v>119</v>
@@ -1906,7 +1962,7 @@
         <v>181</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D28" t="s">
         <v>119</v>
@@ -1923,10 +1979,10 @@
     </row>
     <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E29" t="s">
         <v>140</v>
@@ -1943,7 +1999,7 @@
         <v>94</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="E30" t="s">
         <v>168</v>
@@ -1960,7 +2016,7 @@
         <v>95</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D31" t="s">
         <v>119</v>
@@ -1980,15 +2036,15 @@
         <v>177</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D33" t="s">
         <v>119</v>
@@ -2005,10 +2061,10 @@
     </row>
     <row r="34" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="E34" t="s">
         <v>168</v>
@@ -2022,10 +2078,10 @@
     </row>
     <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E35" t="s">
         <v>168</v>
@@ -2039,10 +2095,10 @@
     </row>
     <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="E36" t="s">
         <v>168</v>
@@ -2056,10 +2112,10 @@
     </row>
     <row r="37" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="E37" t="s">
         <v>168</v>
@@ -2076,7 +2132,7 @@
         <v>178</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D38" t="s">
         <v>120</v>
@@ -2093,10 +2149,10 @@
     </row>
     <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D39" t="s">
         <v>120</v>
@@ -2113,10 +2169,10 @@
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D40" t="s">
         <v>120</v>
@@ -2133,10 +2189,10 @@
     </row>
     <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D41" t="s">
         <v>120</v>
@@ -2153,10 +2209,10 @@
     </row>
     <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D42" t="s">
         <v>120</v>
@@ -2173,7 +2229,7 @@
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B43" s="16" t="s">
         <v>186</v>
@@ -2193,7 +2249,7 @@
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B44" s="16" t="s">
         <v>187</v>
@@ -2253,7 +2309,7 @@
     </row>
     <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="B47" s="16" t="s">
         <v>101</v>
@@ -2273,7 +2329,7 @@
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B48" s="16" t="s">
         <v>102</v>
@@ -2293,7 +2349,7 @@
     </row>
     <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B49" s="16" t="s">
         <v>103</v>
@@ -2367,7 +2423,7 @@
         <v>189</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D53" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
Construction of assurance argument for HL-1-3-1 and associated detection and recording of issues.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878297AD-C290-6A44-A429-4B3A8ECF2DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C2FC27-33C9-4540-82A3-2B9C0B5CCCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
@@ -843,13 +843,13 @@
     <t>HL-1-3-3</t>
   </si>
   <si>
-    <t>Zone geometry applied is isufficiently correct and accurate</t>
-  </si>
-  <si>
-    <t>Computation of existing zone violations is correct and accurate with respect to a vehicle state event</t>
-  </si>
-  <si>
-    <t>Computation of imminent zone violations is correct and accurate with respect to vehicle state events and linear immediate trajectory</t>
+    <t>Th zone geometry applied is sufficiently correct and accurate</t>
+  </si>
+  <si>
+    <t>Computation of existing zone violations is correct and accurate with respect to a vehicle state event and stored zone geometry</t>
+  </si>
+  <si>
+    <t>Computation of imminent zone violations is correct and accurate with respect to vehicle state events and linear immediate trajectory and stored zone geometry</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Updates to argument for HL-1-2.gsn with tweeks of reuiqrements. Labelling of HL1-2.gsn with requirements where claims use requirements. Note of where argument diverges. Improved fidelity architecture diagram.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86C2FC27-33C9-4540-82A3-2B9C0B5CCCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3545CFC-5900-0140-BB35-5BBC62183FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="272">
   <si>
     <t>Name</t>
   </si>
@@ -714,9 +714,6 @@
     <t>SR-4-3-2-1</t>
   </si>
   <si>
-    <t>The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric applied in the RoutePlannerVisbilityService when it calls bFindPointsForAbstractGeometry method</t>
-  </si>
-  <si>
     <t>The ZoneAlertComputer shall store all declared abstract geometries by calling the same bFindPointsForAbstractGeometry function as used by RoutePLannerVisibilityService.</t>
   </si>
   <si>
@@ -759,9 +756,6 @@
     <t>The Zone Alert COmputer assign a unique id to each resulting merged zone created as output of the VisibilityGraph</t>
   </si>
   <si>
-    <t>When all zones are finished being declared by OpenUxAS, rhe service shall perform zone checking, explansion, and merging using the standard defined zone processing semantcs of the RoutePlannerVisbilityService when an Operating Region is declared</t>
-  </si>
-  <si>
     <t xml:space="preserve">The zone service shall expand, merge, and check all zones using the same semantics </t>
   </si>
   <si>
@@ -843,13 +837,25 @@
     <t>HL-1-3-3</t>
   </si>
   <si>
-    <t>Th zone geometry applied is sufficiently correct and accurate</t>
-  </si>
-  <si>
     <t>Computation of existing zone violations is correct and accurate with respect to a vehicle state event and stored zone geometry</t>
   </si>
   <si>
     <t>Computation of imminent zone violations is correct and accurate with respect to vehicle state events and linear immediate trajectory and stored zone geometry</t>
+  </si>
+  <si>
+    <t>The zone geometry applied is sufficiently correct and accurate</t>
+  </si>
+  <si>
+    <t>SR-4-3-2-2</t>
+  </si>
+  <si>
+    <t>The ZoneAlertComputer shall store all computed intermediate polygons returned as success by bFindPointsForAbstractGeomrty as Cboundary objects mapped by zone id, just as RoutePlannerVisiblityService does</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The ZoneAlertComputer shall store zones as  closed irregular polygons in the Cartesian plane with the equivalent analytic geometric computation applied in the RoutePlannerVisbilityService </t>
+  </si>
+  <si>
+    <t>When all zones are finished being declared by OpenUxAS, the service shall perform zone checking, explansion, and merging using the standard defined zone processing semantcs of the RoutePlannerVisbilityService when an Operating Region is declared</t>
   </si>
 </sst>
 </file>
@@ -1378,20 +1384,20 @@
         <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B5" t="s">
         <v>267</v>
@@ -1399,18 +1405,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>263</v>
+      </c>
+      <c r="B6" t="s">
         <v>265</v>
-      </c>
-      <c r="B6" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>264</v>
+      </c>
+      <c r="B7" t="s">
         <v>266</v>
-      </c>
-      <c r="B7" t="s">
-        <v>269</v>
       </c>
     </row>
   </sheetData>
@@ -1420,7 +1426,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34AC7C05-FC71-F749-BB41-F1A5141E29DB}">
-  <dimension ref="A1:G99"/>
+  <dimension ref="A1:G100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -1711,7 +1717,7 @@
         <v>158</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D15" t="s">
         <v>119</v>
@@ -1751,7 +1757,7 @@
         <v>160</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>224</v>
+        <v>270</v>
       </c>
       <c r="D17" t="s">
         <v>120</v>
@@ -1771,7 +1777,7 @@
         <v>223</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D18" t="s">
         <v>120</v>
@@ -1786,55 +1792,58 @@
         <v>167</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
+        <v>268</v>
+      </c>
+      <c r="B19" s="16" t="s">
+        <v>269</v>
+      </c>
+      <c r="D19" t="s">
+        <v>120</v>
+      </c>
+      <c r="E19" t="s">
+        <v>168</v>
+      </c>
+      <c r="F19" t="s">
+        <v>120</v>
+      </c>
+      <c r="G19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B20" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C20" t="s">
         <v>84</v>
       </c>
-      <c r="D19" t="s">
-        <v>119</v>
-      </c>
-      <c r="E19" t="s">
-        <v>140</v>
-      </c>
-      <c r="F19" t="s">
-        <v>119</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="D20" t="s">
+        <v>119</v>
+      </c>
+      <c r="E20" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" t="s">
+        <v>119</v>
+      </c>
+      <c r="G20" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="17" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="21" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>86</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B21" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="D20" t="s">
-        <v>119</v>
-      </c>
-      <c r="E20" t="s">
-        <v>140</v>
-      </c>
-      <c r="F20" t="s">
-        <v>119</v>
-      </c>
-      <c r="G20" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B21" s="16" t="s">
-        <v>169</v>
+      <c r="D21" t="s">
+        <v>119</v>
       </c>
       <c r="E21" t="s">
         <v>140</v>
@@ -1846,143 +1855,143 @@
         <v>144</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>169</v>
+      </c>
+      <c r="E22" t="s">
+        <v>140</v>
+      </c>
+      <c r="F22" t="s">
+        <v>119</v>
+      </c>
+      <c r="G22" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>170</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B23" s="16" t="s">
         <v>173</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D23" t="s">
         <v>126</v>
       </c>
-      <c r="E22" t="s">
-        <v>140</v>
-      </c>
-      <c r="F22" t="s">
-        <v>119</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="E23" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" t="s">
+        <v>119</v>
+      </c>
+      <c r="G23" t="s">
         <v>166</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>171</v>
-      </c>
-      <c r="B23" s="16" t="s">
-        <v>175</v>
-      </c>
-      <c r="D23" t="s">
-        <v>119</v>
-      </c>
-      <c r="E23" t="s">
-        <v>140</v>
-      </c>
-      <c r="F23" t="s">
-        <v>119</v>
-      </c>
-      <c r="G23" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>258</v>
+        <v>175</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E24" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="F24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G24" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>256</v>
+      </c>
+      <c r="D25" t="s">
+        <v>120</v>
+      </c>
+      <c r="E25" t="s">
+        <v>168</v>
+      </c>
+      <c r="F25" t="s">
+        <v>120</v>
+      </c>
+      <c r="G25" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
         <v>90</v>
       </c>
-      <c r="B25" s="16" t="s">
-        <v>240</v>
-      </c>
-      <c r="E25" t="s">
-        <v>140</v>
-      </c>
-      <c r="F25" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="85" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="B26" s="16" t="s">
+        <v>238</v>
+      </c>
+      <c r="E26" t="s">
+        <v>140</v>
+      </c>
+      <c r="F26" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
         <v>93</v>
       </c>
-      <c r="B26" s="16" t="s">
-        <v>239</v>
-      </c>
-      <c r="D26" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" t="s">
-        <v>140</v>
-      </c>
-      <c r="F26" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="B27" s="16" t="s">
+        <v>271</v>
+      </c>
+      <c r="D27" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
         <v>180</v>
       </c>
-      <c r="B27" s="16" t="s">
+      <c r="B28" s="16" t="s">
         <v>92</v>
       </c>
-      <c r="D27" t="s">
-        <v>119</v>
-      </c>
-      <c r="E27" t="s">
-        <v>140</v>
-      </c>
-      <c r="F27" t="s">
-        <v>119</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="D28" t="s">
+        <v>119</v>
+      </c>
+      <c r="E28" t="s">
+        <v>140</v>
+      </c>
+      <c r="F28" t="s">
+        <v>119</v>
+      </c>
+      <c r="G28" t="s">
         <v>144</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>181</v>
-      </c>
-      <c r="B28" s="16" t="s">
-        <v>256</v>
-      </c>
-      <c r="D28" t="s">
-        <v>119</v>
-      </c>
-      <c r="E28" t="s">
-        <v>140</v>
-      </c>
-      <c r="F28" t="s">
-        <v>119</v>
-      </c>
-      <c r="G28" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>257</v>
+        <v>181</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>241</v>
+        <v>254</v>
+      </c>
+      <c r="D29" t="s">
+        <v>119</v>
       </c>
       <c r="E29" t="s">
         <v>140</v>
@@ -1991,35 +2000,32 @@
         <v>119</v>
       </c>
       <c r="G29" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>94</v>
+        <v>255</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>252</v>
+        <v>239</v>
       </c>
       <c r="E30" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="F30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G30" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="D31" t="s">
-        <v>119</v>
+        <v>250</v>
       </c>
       <c r="E31" t="s">
         <v>168</v>
@@ -2031,40 +2037,43 @@
         <v>182</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>177</v>
+        <v>95</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>228</v>
+        <v>225</v>
+      </c>
+      <c r="D32" t="s">
+        <v>119</v>
+      </c>
+      <c r="E32" t="s">
+        <v>168</v>
+      </c>
+      <c r="F32" t="s">
+        <v>120</v>
+      </c>
+      <c r="G32" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>229</v>
+        <v>177</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>233</v>
-      </c>
-      <c r="D33" t="s">
-        <v>119</v>
-      </c>
-      <c r="E33" t="s">
-        <v>168</v>
-      </c>
-      <c r="F33" t="s">
-        <v>120</v>
-      </c>
-      <c r="G33" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>234</v>
+        <v>232</v>
+      </c>
+      <c r="D34" t="s">
+        <v>119</v>
       </c>
       <c r="E34" t="s">
         <v>168</v>
@@ -2076,12 +2085,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E35" t="s">
         <v>168</v>
@@ -2093,12 +2102,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="E36" t="s">
         <v>168</v>
@@ -2110,12 +2119,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="E37" t="s">
         <v>168</v>
@@ -2129,13 +2138,10 @@
     </row>
     <row r="38" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>178</v>
+        <v>236</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>242</v>
-      </c>
-      <c r="D38" t="s">
-        <v>120</v>
+        <v>235</v>
       </c>
       <c r="E38" t="s">
         <v>168</v>
@@ -2147,12 +2153,12 @@
         <v>182</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>243</v>
+        <v>178</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D39" t="s">
         <v>120</v>
@@ -2169,10 +2175,10 @@
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
       <c r="D40" t="s">
         <v>120</v>
@@ -2189,10 +2195,10 @@
     </row>
     <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D41" t="s">
         <v>120</v>
@@ -2209,10 +2215,10 @@
     </row>
     <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="D42" t="s">
         <v>120</v>
@@ -2229,10 +2235,10 @@
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>186</v>
+        <v>249</v>
       </c>
       <c r="D43" t="s">
         <v>120</v>
@@ -2249,10 +2255,10 @@
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D44" t="s">
         <v>120</v>
@@ -2269,30 +2275,30 @@
     </row>
     <row r="45" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
+        <v>253</v>
+      </c>
+      <c r="B45" s="16" t="s">
+        <v>187</v>
+      </c>
+      <c r="D45" t="s">
+        <v>120</v>
+      </c>
+      <c r="E45" t="s">
+        <v>168</v>
+      </c>
+      <c r="F45" t="s">
+        <v>120</v>
+      </c>
+      <c r="G45" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
         <v>183</v>
       </c>
-      <c r="B45" s="16" t="s">
+      <c r="B46" s="16" t="s">
         <v>100</v>
-      </c>
-      <c r="D45" t="s">
-        <v>119</v>
-      </c>
-      <c r="E45" t="s">
-        <v>140</v>
-      </c>
-      <c r="F45" t="s">
-        <v>119</v>
-      </c>
-      <c r="G45" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>184</v>
-      </c>
-      <c r="B46" s="16" t="s">
-        <v>185</v>
       </c>
       <c r="D46" t="s">
         <v>119</v>
@@ -2307,15 +2313,15 @@
         <v>166</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>248</v>
+        <v>184</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>101</v>
+        <v>185</v>
       </c>
       <c r="D47" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="E47" t="s">
         <v>140</v>
@@ -2329,10 +2335,10 @@
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D48" t="s">
         <v>127</v>
@@ -2349,10 +2355,10 @@
     </row>
     <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D49" t="s">
         <v>127</v>
@@ -2367,123 +2373,123 @@
         <v>166</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
+        <v>248</v>
+      </c>
+      <c r="B50" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="D50" t="s">
+        <v>127</v>
+      </c>
+      <c r="E50" t="s">
+        <v>140</v>
+      </c>
+      <c r="F50" t="s">
+        <v>119</v>
+      </c>
+      <c r="G50" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
         <v>96</v>
       </c>
-      <c r="B50" s="16" t="s">
+      <c r="B51" s="16" t="s">
         <v>205</v>
       </c>
-      <c r="D50" t="s">
-        <v>119</v>
-      </c>
-      <c r="E50" t="s">
-        <v>140</v>
-      </c>
-      <c r="F50" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="D51" t="s">
+        <v>119</v>
+      </c>
+      <c r="E51" t="s">
+        <v>140</v>
+      </c>
+      <c r="F51" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
         <v>91</v>
       </c>
-      <c r="B51" s="16" t="s">
+      <c r="B52" s="16" t="s">
         <v>188</v>
       </c>
-      <c r="E51" t="s">
-        <v>140</v>
-      </c>
-      <c r="F51" t="s">
-        <v>119</v>
-      </c>
-      <c r="G51" t="s">
+      <c r="E52" t="s">
+        <v>140</v>
+      </c>
+      <c r="F52" t="s">
+        <v>119</v>
+      </c>
+      <c r="G52" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+    <row r="53" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
         <v>97</v>
       </c>
-      <c r="B52" s="16" t="s">
+      <c r="B53" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="D52" t="s">
-        <v>119</v>
-      </c>
-      <c r="E52" t="s">
-        <v>140</v>
-      </c>
-      <c r="F52" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="D53" t="s">
+        <v>119</v>
+      </c>
+      <c r="E53" t="s">
+        <v>140</v>
+      </c>
+      <c r="F53" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>189</v>
       </c>
-      <c r="B53" s="16" t="s">
-        <v>259</v>
-      </c>
-      <c r="D53" t="s">
-        <v>119</v>
-      </c>
-      <c r="E53" t="s">
-        <v>140</v>
-      </c>
-      <c r="F53" t="s">
-        <v>119</v>
-      </c>
-      <c r="G53" t="s">
+      <c r="B54" s="16" t="s">
+        <v>257</v>
+      </c>
+      <c r="D54" t="s">
+        <v>119</v>
+      </c>
+      <c r="E54" t="s">
+        <v>140</v>
+      </c>
+      <c r="F54" t="s">
+        <v>119</v>
+      </c>
+      <c r="G54" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="54" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+    <row r="55" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>190</v>
       </c>
-      <c r="B54" s="16" t="s">
+      <c r="B55" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="D54" t="s">
-        <v>119</v>
-      </c>
-      <c r="E54" t="s">
-        <v>140</v>
-      </c>
-      <c r="F54" t="s">
-        <v>119</v>
-      </c>
-      <c r="G54" t="s">
+      <c r="D55" t="s">
+        <v>119</v>
+      </c>
+      <c r="E55" t="s">
+        <v>140</v>
+      </c>
+      <c r="F55" t="s">
+        <v>119</v>
+      </c>
+      <c r="G55" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="55" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
+    <row r="56" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
         <v>192</v>
       </c>
-      <c r="B55" s="16" t="s">
+      <c r="B56" s="16" t="s">
         <v>129</v>
-      </c>
-      <c r="D55" t="s">
-        <v>120</v>
-      </c>
-      <c r="E55" t="s">
-        <v>168</v>
-      </c>
-      <c r="F55" t="s">
-        <v>120</v>
-      </c>
-      <c r="G55" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
-        <v>194</v>
-      </c>
-      <c r="B56" s="16" t="s">
-        <v>130</v>
       </c>
       <c r="D56" t="s">
         <v>120</v>
@@ -2498,12 +2504,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D57" t="s">
         <v>120</v>
@@ -2520,10 +2526,13 @@
     </row>
     <row r="58" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>197</v>
+        <v>132</v>
+      </c>
+      <c r="D58" t="s">
+        <v>120</v>
       </c>
       <c r="E58" t="s">
         <v>168</v>
@@ -2535,15 +2544,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A59" s="14" t="s">
-        <v>198</v>
+    <row r="59" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>196</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="D59" t="s">
-        <v>120</v>
+        <v>197</v>
       </c>
       <c r="E59" t="s">
         <v>168</v>
@@ -2555,12 +2561,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="102" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D60" t="s">
         <v>120</v>
@@ -2575,12 +2581,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>199</v>
+        <v>133</v>
       </c>
       <c r="D61" t="s">
         <v>120</v>
@@ -2595,12 +2601,15 @@
         <v>193</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ht="153" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>134</v>
+        <v>199</v>
+      </c>
+      <c r="D62" t="s">
+        <v>120</v>
       </c>
       <c r="E62" t="s">
         <v>168</v>
@@ -2612,12 +2621,12 @@
         <v>193</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="102" x14ac:dyDescent="0.2">
-      <c r="A63" t="s">
-        <v>202</v>
+    <row r="63" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A63" s="14" t="s">
+        <v>201</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>203</v>
+        <v>134</v>
       </c>
       <c r="E63" t="s">
         <v>168</v>
@@ -2629,29 +2638,29 @@
         <v>193</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>98</v>
+        <v>202</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>106</v>
+        <v>203</v>
       </c>
       <c r="E64" t="s">
-        <v>140</v>
+        <v>168</v>
       </c>
       <c r="F64" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G64" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>206</v>
+        <v>98</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E65" t="s">
         <v>140</v>
@@ -2665,10 +2674,10 @@
     </row>
     <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E66" t="s">
         <v>140</v>
@@ -2682,10 +2691,10 @@
     </row>
     <row r="67" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E67" t="s">
         <v>140</v>
@@ -2699,10 +2708,10 @@
     </row>
     <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E68" t="s">
         <v>140</v>
@@ -2714,12 +2723,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E69" t="s">
         <v>140</v>
@@ -2731,12 +2740,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B70" s="16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E70" t="s">
         <v>140</v>
@@ -2748,12 +2757,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E71" t="s">
         <v>140</v>
@@ -2765,12 +2774,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="E72" t="s">
         <v>140</v>
@@ -2784,10 +2793,10 @@
     </row>
     <row r="73" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E73" t="s">
         <v>140</v>
@@ -2799,12 +2808,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E74" t="s">
         <v>140</v>
@@ -2818,10 +2827,10 @@
     </row>
     <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>99</v>
+        <v>215</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E75" t="s">
         <v>140</v>
@@ -2833,15 +2842,12 @@
         <v>191</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B76" s="16" t="s">
-        <v>179</v>
-      </c>
-      <c r="D76" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E76" t="s">
         <v>140</v>
@@ -2850,32 +2856,35 @@
         <v>119</v>
       </c>
       <c r="G76" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>161</v>
+        <v>104</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>163</v>
+        <v>179</v>
+      </c>
+      <c r="D77" t="s">
+        <v>119</v>
       </c>
       <c r="E77" t="s">
-        <v>168</v>
+        <v>140</v>
       </c>
       <c r="F77" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G77" t="s">
-        <v>182</v>
+        <v>166</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E78" t="s">
         <v>168</v>
@@ -2884,11 +2893,25 @@
         <v>120</v>
       </c>
       <c r="G78" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>162</v>
+      </c>
+      <c r="B79" s="16" t="s">
+        <v>164</v>
+      </c>
+      <c r="E79" t="s">
+        <v>168</v>
+      </c>
+      <c r="F79" t="s">
+        <v>120</v>
+      </c>
+      <c r="G79" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B79" s="16"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B80" s="16"/>
@@ -2900,7 +2923,7 @@
       <c r="B82" s="16"/>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B83" s="18"/>
+      <c r="B83" s="16"/>
     </row>
     <row r="84" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B84" s="18"/>
@@ -2909,10 +2932,10 @@
       <c r="B85" s="18"/>
     </row>
     <row r="86" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B86" s="16"/>
+      <c r="B86" s="18"/>
     </row>
     <row r="87" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B87" s="18"/>
+      <c r="B87" s="16"/>
     </row>
     <row r="88" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B88" s="18"/>
@@ -2925,13 +2948,13 @@
     </row>
     <row r="91" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B91" s="18"/>
-      <c r="C91" s="13"/>
     </row>
     <row r="92" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B92" s="16"/>
+      <c r="B92" s="18"/>
+      <c r="C92" s="13"/>
     </row>
     <row r="93" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B93" s="18"/>
+      <c r="B93" s="16"/>
     </row>
     <row r="94" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B94" s="18"/>
@@ -2949,7 +2972,10 @@
       <c r="B98" s="18"/>
     </row>
     <row r="99" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B99" s="16"/>
+      <c r="B99" s="18"/>
+    </row>
+    <row r="100" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B100" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Argument updates moving towards assurance solution map.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3545CFC-5900-0140-BB35-5BBC62183FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0C6977-2648-BE41-86AF-195264B88B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="550" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="276">
   <si>
     <t>Name</t>
   </si>
@@ -816,18 +816,12 @@
     <t>The zone alert service shall respond to a received vehicle state by correctly determining whether a violation exists between the received vehicle state and each merged zone</t>
   </si>
   <si>
-    <t>The service shal utilize the same semantics for zone geometry as RoutePlannerVisibilityService</t>
-  </si>
-  <si>
     <t xml:space="preserve">The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics </t>
   </si>
   <si>
     <t>HL-1-3</t>
   </si>
   <si>
-    <t>The service shall compute zone violations against zone semantics both correctly and accurately</t>
-  </si>
-  <si>
     <t>HL-1-3-1</t>
   </si>
   <si>
@@ -856,6 +850,24 @@
   </si>
   <si>
     <t>When all zones are finished being declared by OpenUxAS, the service shall perform zone checking, explansion, and merging using the standard defined zone processing semantcs of the RoutePlannerVisbilityService when an Operating Region is declared</t>
+  </si>
+  <si>
+    <t>The service shall compute zone violations from vehicle state reports against zone geometry both correctly and accurately.</t>
+  </si>
+  <si>
+    <t>The service shall compute and apply zones of the same geometry computed and applied by the RoutePlannerVisibilityService.</t>
+  </si>
+  <si>
+    <t>The service shall correctly declare all zones it constructs for zone alerting in a timely manner before mission start</t>
+  </si>
+  <si>
+    <t>HL-1-4</t>
+  </si>
+  <si>
+    <t>HL-1-5</t>
+  </si>
+  <si>
+    <t>The service shall correctly report all computed zone violations.</t>
   </si>
 </sst>
 </file>
@@ -1357,7 +1369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FDF8AA6-5D75-9940-86F4-A0A21993176A}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="45.5" customWidth="1"/>
@@ -1384,39 +1396,55 @@
         <v>137</v>
       </c>
       <c r="B3" t="s">
-        <v>258</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B4" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>261</v>
+      </c>
+      <c r="B6" t="s">
         <v>263</v>
-      </c>
-      <c r="B6" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>262</v>
+      </c>
+      <c r="B7" t="s">
         <v>264</v>
       </c>
-      <c r="B7" t="s">
-        <v>266</v>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>273</v>
+      </c>
+      <c r="B8" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>274</v>
+      </c>
+      <c r="B9" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -1717,7 +1745,7 @@
         <v>158</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D15" t="s">
         <v>119</v>
@@ -1757,7 +1785,7 @@
         <v>160</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D17" t="s">
         <v>120</v>
@@ -1794,10 +1822,10 @@
     </row>
     <row r="19" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="D19" t="s">
         <v>120</v>
@@ -1951,7 +1979,7 @@
         <v>93</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="D27" t="s">
         <v>119</v>

</xml_diff>

<commit_message>
Finished up initial draft of assurance argument for the Zone Alert Service.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F0C6977-2648-BE41-86AF-195264B88B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3487210-1F6B-8B41-91CB-1A83AA1DF9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1060" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="17500" yWindow="2860" windowWidth="30580" windowHeight="19520" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
@@ -261,9 +261,6 @@
     <t>HL-1</t>
   </si>
   <si>
-    <t>Provide an OpenUxAS service to make OpenUxAS systems aware of potential for future zone violations by vehicles based on zone and vehicle positinos and vehicle behavior</t>
-  </si>
-  <si>
     <t>The service shall report and error and terminate if an acceptable time window is not defined in configuration parameters.</t>
   </si>
   <si>
@@ -447,15 +444,9 @@
     <t>The zone alert computer shall compute the position and time of a detected existing zone violation between a vehicle's stated position and a merged zone as the stated vehicle position and time of the vehicle state report.</t>
   </si>
   <si>
-    <t>OpenUxAS shall be aware of existing zone violations by vehicles to usefully avoiid/recover/accept imminent and existing zone violations.</t>
-  </si>
-  <si>
     <t>HL-1-1</t>
   </si>
   <si>
-    <t>HL-1-2</t>
-  </si>
-  <si>
     <t>The service shall proceed initialization on parameters by by listening for and recording information about the OpenUxAS missions environment and actors</t>
   </si>
   <si>
@@ -819,27 +810,6 @@
     <t xml:space="preserve">The service shall respond to received zone declaration messages by transforming and storing the zones into polygons in a cartesian plane with equivalent analytic geometry to that of RoutePlanner semantics </t>
   </si>
   <si>
-    <t>HL-1-3</t>
-  </si>
-  <si>
-    <t>HL-1-3-1</t>
-  </si>
-  <si>
-    <t>HL-1-3-2</t>
-  </si>
-  <si>
-    <t>HL-1-3-3</t>
-  </si>
-  <si>
-    <t>Computation of existing zone violations is correct and accurate with respect to a vehicle state event and stored zone geometry</t>
-  </si>
-  <si>
-    <t>Computation of imminent zone violations is correct and accurate with respect to vehicle state events and linear immediate trajectory and stored zone geometry</t>
-  </si>
-  <si>
-    <t>The zone geometry applied is sufficiently correct and accurate</t>
-  </si>
-  <si>
     <t>SR-4-3-2-2</t>
   </si>
   <si>
@@ -852,22 +822,52 @@
     <t>When all zones are finished being declared by OpenUxAS, the service shall perform zone checking, explansion, and merging using the standard defined zone processing semantcs of the RoutePlannerVisbilityService when an Operating Region is declared</t>
   </si>
   <si>
-    <t>The service shall compute zone violations from vehicle state reports against zone geometry both correctly and accurately.</t>
-  </si>
-  <si>
     <t>The service shall compute and apply zones of the same geometry computed and applied by the RoutePlannerVisibilityService.</t>
   </si>
   <si>
     <t>The service shall correctly declare all zones it constructs for zone alerting in a timely manner before mission start</t>
   </si>
   <si>
-    <t>HL-1-4</t>
-  </si>
-  <si>
-    <t>HL-1-5</t>
-  </si>
-  <si>
-    <t>The service shall correctly report all computed zone violations.</t>
+    <t>Provide an OpenUxAS service to make OpenUxAS systems aware of potential for future zone violations by vehicles based on zone and vehicle positions and vehicle behavior</t>
+  </si>
+  <si>
+    <t>HL-1-1-1</t>
+  </si>
+  <si>
+    <t>HL-1-1-2</t>
+  </si>
+  <si>
+    <t>HL-1-1-2-1</t>
+  </si>
+  <si>
+    <t>HL-1-1-2-2</t>
+  </si>
+  <si>
+    <t>HL-1-1-2-3</t>
+  </si>
+  <si>
+    <t>HL-1-1-3</t>
+  </si>
+  <si>
+    <t>The service shall correctly and accurately report existing zone violations</t>
+  </si>
+  <si>
+    <t>The service shall correctly and accurately report imminent zone violations</t>
+  </si>
+  <si>
+    <t>The service shall interpet declared zones in the same manner as the RoutePlannerVisibilityService.</t>
+  </si>
+  <si>
+    <t>OpenUxAS shall be aware of existing zone violations by vehicles to usefully avoid/recover/accept imminent and existing zone violations.</t>
+  </si>
+  <si>
+    <t>The service correctly and accurately report zone violations from vehicle state reports and computed zone geometry</t>
+  </si>
+  <si>
+    <t>HL-1-1-2-4</t>
+  </si>
+  <si>
+    <t>The zone geometry applied is sufficiently correct and accurate.</t>
   </si>
 </sst>
 </file>
@@ -1380,20 +1380,20 @@
         <v>72</v>
       </c>
       <c r="B1" t="s">
-        <v>135</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>262</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>137</v>
+        <v>263</v>
       </c>
       <c r="B3" t="s">
         <v>271</v>
@@ -1401,50 +1401,50 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="B4" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="B5" t="s">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B6" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B7" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B8" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B9" t="s">
-        <v>275</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -1474,1471 +1474,1471 @@
         <v>71</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D1" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F1" s="12" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="52" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G3" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E6" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E7" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G7" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E8" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G8" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E9" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G9" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F10" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="G10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F11" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E13" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F13" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G13" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="D14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E14" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G14" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G15" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E16" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F16" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G16" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="D17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E17" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E18" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="D19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G19" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="C20" t="s">
         <v>83</v>
       </c>
-      <c r="C20" t="s">
-        <v>84</v>
-      </c>
       <c r="D20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E20" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G20" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D21" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E21" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F21" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G21" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E22" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G22" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="16" t="s">
         <v>170</v>
       </c>
-      <c r="B23" s="16" t="s">
-        <v>173</v>
-      </c>
       <c r="D23" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E23" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G23" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E24" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G24" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E25" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G25" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E26" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="D27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E28" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G28" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F29" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G29" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E30" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G30" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="E31" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G31" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D32" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E32" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F32" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G32" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D34" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F34" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G34" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E35" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F35" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G35" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F36" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G36" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E37" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G37" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="E38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G38" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E39" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G39" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E40" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F40" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G40" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E41" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F41" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G41" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E42" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F42" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G42" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D43" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E43" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F43" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G43" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D44" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E44" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F44" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G44" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D45" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E45" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F45" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G45" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D46" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E46" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F46" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G46" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E47" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F47" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G47" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D48" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E48" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F48" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G48" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E49" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F49" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G49" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E50" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F50" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G50" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="D51" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E51" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F51" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B52" s="16" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="E52" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F52" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G52" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="53" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B53" s="16" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D53" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E53" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F53" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="54" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B54" s="16" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D54" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E54" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F54" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G54" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B55" s="16" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D55" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E55" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F55" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G55" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B56" s="16" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E56" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F56" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G56" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B57" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E57" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F57" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G57" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B58" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D58" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E58" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F58" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G58" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E59" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F59" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G59" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="60" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A60" s="14" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E60" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G60" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="61" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A61" s="14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D61" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E61" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F61" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G61" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="153" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E62" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G62" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A63" s="14" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E63" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F63" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G63" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="64" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E64" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F64" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G64" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E65" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F65" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G65" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E66" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F66" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G66" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E67" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F67" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G67" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E68" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F68" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G68" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="69" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E69" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F69" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G69" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B70" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E70" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F70" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G70" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E71" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F71" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G71" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E72" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F72" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G72" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E73" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F73" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G73" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="74" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E74" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F74" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G74" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E75" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F75" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G75" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B76" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E76" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F76" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G76" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D77" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E77" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F77" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G77" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E78" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F78" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G78" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B79" s="16" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E79" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="F79" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G79" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.2">
@@ -3018,35 +3018,35 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated issues, requirements, solutionExploration for issue 49.
</commit_message>
<xml_diff>
--- a/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
+++ b/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/requirements.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Dependable/Contracts/ASTRA/Deliverables/OpenUxAS-ZoneAlert/doc/assurance/ZoneAlertService/3-Specification/A-Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3487210-1F6B-8B41-91CB-1A83AA1DF9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83BDD75F-AD17-7040-9CA0-FEEF9F187E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17500" yWindow="2860" windowWidth="30580" windowHeight="19520" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
+    <workbookView xWindow="5260" yWindow="2860" windowWidth="30580" windowHeight="19520" activeTab="1" xr2:uid="{A76FD67C-FD1A-274E-A8A0-8B595CED0661}"/>
   </bookViews>
   <sheets>
     <sheet name="HighLevelRequirements" sheetId="6" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="280">
   <si>
     <t>Name</t>
   </si>
@@ -868,6 +868,18 @@
   </si>
   <si>
     <t>The zone geometry applied is sufficiently correct and accurate.</t>
+  </si>
+  <si>
+    <t>SR-6-2-3</t>
+  </si>
+  <si>
+    <t>The Zone Alert Computer shall expand and merge zones without using Zone Padding. Zone padding shall not be used as it offsets routes from the edge of zones, and we are not offseting zone edges, instead reporting violations of exact zone boundaries.</t>
+  </si>
+  <si>
+    <t>SR-6-2-3-1</t>
+  </si>
+  <si>
+    <t>The zone alert computer shall store received zones with a padding value of zero regardless of what padding for the zone is received in its declaration message</t>
   </si>
 </sst>
 </file>
@@ -1454,7 +1466,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34AC7C05-FC71-F749-BB41-F1A5141E29DB}">
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -2181,35 +2193,29 @@
         <v>179</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ht="85" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>175</v>
+        <v>276</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>237</v>
-      </c>
-      <c r="D39" t="s">
-        <v>119</v>
+        <v>277</v>
       </c>
       <c r="E39" t="s">
         <v>165</v>
       </c>
       <c r="F39" t="s">
-        <v>119</v>
+        <v>165</v>
       </c>
       <c r="G39" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>238</v>
+        <v>278</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>234</v>
-      </c>
-      <c r="D40" t="s">
-        <v>119</v>
+        <v>279</v>
       </c>
       <c r="E40" t="s">
         <v>165</v>
@@ -2218,15 +2224,15 @@
         <v>119</v>
       </c>
       <c r="G40" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>239</v>
+        <v>175</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="D41" t="s">
         <v>119</v>
@@ -2243,10 +2249,10 @@
     </row>
     <row r="42" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="D42" t="s">
         <v>119</v>
@@ -2263,10 +2269,10 @@
     </row>
     <row r="43" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D43" t="s">
         <v>119</v>
@@ -2283,10 +2289,10 @@
     </row>
     <row r="44" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="B44" s="16" t="s">
-        <v>183</v>
+        <v>241</v>
       </c>
       <c r="D44" t="s">
         <v>119</v>
@@ -2303,10 +2309,10 @@
     </row>
     <row r="45" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="B45" s="16" t="s">
-        <v>184</v>
+        <v>246</v>
       </c>
       <c r="D45" t="s">
         <v>119</v>
@@ -2323,53 +2329,53 @@
     </row>
     <row r="46" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>180</v>
+        <v>249</v>
       </c>
       <c r="B46" s="16" t="s">
-        <v>99</v>
+        <v>183</v>
       </c>
       <c r="D46" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E46" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="F46" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G46" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>181</v>
+        <v>250</v>
       </c>
       <c r="B47" s="16" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D47" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E47" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="F47" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G47" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="48" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>243</v>
+        <v>180</v>
       </c>
       <c r="B48" s="16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D48" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E48" t="s">
         <v>137</v>
@@ -2381,15 +2387,15 @@
         <v>163</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>244</v>
+        <v>181</v>
       </c>
       <c r="B49" s="16" t="s">
-        <v>101</v>
+        <v>182</v>
       </c>
       <c r="D49" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="E49" t="s">
         <v>137</v>
@@ -2403,10 +2409,10 @@
     </row>
     <row r="50" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="D50" t="s">
         <v>126</v>
@@ -2421,84 +2427,87 @@
         <v>163</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>95</v>
+        <v>244</v>
       </c>
       <c r="B51" s="16" t="s">
-        <v>202</v>
+        <v>101</v>
       </c>
       <c r="D51" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="E51" t="s">
         <v>137</v>
       </c>
       <c r="F51" t="s">
         <v>118</v>
+      </c>
+      <c r="G51" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>245</v>
+      </c>
+      <c r="B52" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="D52" t="s">
+        <v>126</v>
+      </c>
+      <c r="E52" t="s">
+        <v>137</v>
+      </c>
+      <c r="F52" t="s">
+        <v>118</v>
+      </c>
+      <c r="G52" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>95</v>
+      </c>
+      <c r="B53" s="16" t="s">
+        <v>202</v>
+      </c>
+      <c r="D53" t="s">
+        <v>118</v>
+      </c>
+      <c r="E53" t="s">
+        <v>137</v>
+      </c>
+      <c r="F53" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
         <v>90</v>
       </c>
-      <c r="B52" s="16" t="s">
+      <c r="B54" s="16" t="s">
         <v>185</v>
       </c>
-      <c r="E52" t="s">
-        <v>137</v>
-      </c>
-      <c r="F52" t="s">
-        <v>118</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="E54" t="s">
+        <v>137</v>
+      </c>
+      <c r="F54" t="s">
+        <v>118</v>
+      </c>
+      <c r="G54" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+    <row r="55" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
         <v>96</v>
       </c>
-      <c r="B53" s="16" t="s">
+      <c r="B55" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="D53" t="s">
-        <v>118</v>
-      </c>
-      <c r="E53" t="s">
-        <v>137</v>
-      </c>
-      <c r="F53" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="51" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
-        <v>186</v>
-      </c>
-      <c r="B54" s="16" t="s">
-        <v>254</v>
-      </c>
-      <c r="D54" t="s">
-        <v>118</v>
-      </c>
-      <c r="E54" t="s">
-        <v>137</v>
-      </c>
-      <c r="F54" t="s">
-        <v>118</v>
-      </c>
-      <c r="G54" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>187</v>
-      </c>
-      <c r="B55" s="16" t="s">
-        <v>127</v>
-      </c>
       <c r="D55" t="s">
         <v>118</v>
       </c>
@@ -2507,57 +2516,54 @@
       </c>
       <c r="F55" t="s">
         <v>118</v>
-      </c>
-      <c r="G55" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="56" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
+        <v>186</v>
+      </c>
+      <c r="B56" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="D56" t="s">
+        <v>118</v>
+      </c>
+      <c r="E56" t="s">
+        <v>137</v>
+      </c>
+      <c r="F56" t="s">
+        <v>118</v>
+      </c>
+      <c r="G56" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>187</v>
+      </c>
+      <c r="B57" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D57" t="s">
+        <v>118</v>
+      </c>
+      <c r="E57" t="s">
+        <v>137</v>
+      </c>
+      <c r="F57" t="s">
+        <v>118</v>
+      </c>
+      <c r="G57" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
         <v>189</v>
       </c>
-      <c r="B56" s="16" t="s">
+      <c r="B58" s="16" t="s">
         <v>128</v>
-      </c>
-      <c r="D56" t="s">
-        <v>119</v>
-      </c>
-      <c r="E56" t="s">
-        <v>165</v>
-      </c>
-      <c r="F56" t="s">
-        <v>119</v>
-      </c>
-      <c r="G56" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
-        <v>191</v>
-      </c>
-      <c r="B57" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="D57" t="s">
-        <v>119</v>
-      </c>
-      <c r="E57" t="s">
-        <v>165</v>
-      </c>
-      <c r="F57" t="s">
-        <v>119</v>
-      </c>
-      <c r="G57" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="85" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>192</v>
-      </c>
-      <c r="B58" s="16" t="s">
-        <v>131</v>
       </c>
       <c r="D58" t="s">
         <v>119</v>
@@ -2572,12 +2578,15 @@
         <v>190</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B59" s="16" t="s">
-        <v>194</v>
+        <v>129</v>
+      </c>
+      <c r="D59" t="s">
+        <v>119</v>
       </c>
       <c r="E59" t="s">
         <v>165</v>
@@ -2589,12 +2598,12 @@
         <v>190</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="68" x14ac:dyDescent="0.2">
-      <c r="A60" s="14" t="s">
-        <v>195</v>
+    <row r="60" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>192</v>
       </c>
       <c r="B60" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D60" t="s">
         <v>119</v>
@@ -2609,15 +2618,12 @@
         <v>190</v>
       </c>
     </row>
-    <row r="61" spans="1:7" ht="102" x14ac:dyDescent="0.2">
-      <c r="A61" s="14" t="s">
-        <v>201</v>
+    <row r="61" spans="1:7" ht="85" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>193</v>
       </c>
       <c r="B61" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="D61" t="s">
-        <v>119</v>
+        <v>194</v>
       </c>
       <c r="E61" t="s">
         <v>165</v>
@@ -2629,12 +2635,12 @@
         <v>190</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A62" s="14" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B62" s="16" t="s">
-        <v>196</v>
+        <v>130</v>
       </c>
       <c r="D62" t="s">
         <v>119</v>
@@ -2649,12 +2655,15 @@
         <v>190</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A63" s="14" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B63" s="16" t="s">
-        <v>133</v>
+        <v>132</v>
+      </c>
+      <c r="D63" t="s">
+        <v>119</v>
       </c>
       <c r="E63" t="s">
         <v>165</v>
@@ -2666,12 +2675,15 @@
         <v>190</v>
       </c>
     </row>
-    <row r="64" spans="1:7" ht="102" x14ac:dyDescent="0.2">
-      <c r="A64" t="s">
-        <v>199</v>
+    <row r="64" spans="1:7" ht="153" x14ac:dyDescent="0.2">
+      <c r="A64" s="14" t="s">
+        <v>197</v>
       </c>
       <c r="B64" s="16" t="s">
-        <v>200</v>
+        <v>196</v>
+      </c>
+      <c r="D64" t="s">
+        <v>119</v>
       </c>
       <c r="E64" t="s">
         <v>165</v>
@@ -2683,46 +2695,46 @@
         <v>190</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="34" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
-        <v>97</v>
+    <row r="65" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+      <c r="A65" s="14" t="s">
+        <v>198</v>
       </c>
       <c r="B65" s="16" t="s">
-        <v>105</v>
+        <v>133</v>
       </c>
       <c r="E65" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="F65" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G65" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" ht="102" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="B66" s="16" t="s">
-        <v>106</v>
+        <v>200</v>
       </c>
       <c r="E66" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="F66" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G66" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="67" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>204</v>
+        <v>97</v>
       </c>
       <c r="B67" s="16" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E67" t="s">
         <v>137</v>
@@ -2736,10 +2748,10 @@
     </row>
     <row r="68" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B68" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E68" t="s">
         <v>137</v>
@@ -2753,10 +2765,10 @@
     </row>
     <row r="69" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B69" s="16" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E69" t="s">
         <v>137</v>
@@ -2768,12 +2780,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B70" s="16" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E70" t="s">
         <v>137</v>
@@ -2785,12 +2797,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B71" s="16" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="E71" t="s">
         <v>137</v>
@@ -2802,12 +2814,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B72" s="16" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E72" t="s">
         <v>137</v>
@@ -2821,10 +2833,10 @@
     </row>
     <row r="73" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B73" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E73" t="s">
         <v>137</v>
@@ -2836,12 +2848,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="74" spans="1:7" ht="68" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B74" s="16" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E74" t="s">
         <v>137</v>
@@ -2853,12 +2865,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="75" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B75" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E75" t="s">
         <v>137</v>
@@ -2870,12 +2882,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:7" ht="68" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>98</v>
+        <v>211</v>
       </c>
       <c r="B76" s="16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E76" t="s">
         <v>137</v>
@@ -2887,15 +2899,12 @@
         <v>188</v>
       </c>
     </row>
-    <row r="77" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>103</v>
+        <v>212</v>
       </c>
       <c r="B77" s="16" t="s">
-        <v>176</v>
-      </c>
-      <c r="D77" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="E77" t="s">
         <v>137</v>
@@ -2904,93 +2913,124 @@
         <v>118</v>
       </c>
       <c r="G77" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="B78" s="16" t="s">
-        <v>160</v>
+        <v>116</v>
       </c>
       <c r="E78" t="s">
-        <v>165</v>
+        <v>137</v>
       </c>
       <c r="F78" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G78" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="51" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
+        <v>103</v>
+      </c>
+      <c r="B79" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="D79" t="s">
+        <v>118</v>
+      </c>
+      <c r="E79" t="s">
+        <v>137</v>
+      </c>
+      <c r="F79" t="s">
+        <v>118</v>
+      </c>
+      <c r="G79" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>158</v>
+      </c>
+      <c r="B80" s="16" t="s">
+        <v>160</v>
+      </c>
+      <c r="E80" t="s">
+        <v>165</v>
+      </c>
+      <c r="F80" t="s">
+        <v>119</v>
+      </c>
+      <c r="G80" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="51" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>159</v>
       </c>
-      <c r="B79" s="16" t="s">
+      <c r="B81" s="16" t="s">
         <v>161</v>
       </c>
-      <c r="E79" t="s">
+      <c r="E81" t="s">
         <v>165</v>
       </c>
-      <c r="F79" t="s">
-        <v>119</v>
-      </c>
-      <c r="G79" t="s">
+      <c r="F81" t="s">
+        <v>119</v>
+      </c>
+      <c r="G81" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B80" s="16"/>
-    </row>
-    <row r="81" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B81" s="16"/>
-    </row>
-    <row r="82" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B82" s="16"/>
     </row>
-    <row r="83" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B83" s="16"/>
     </row>
-    <row r="84" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B84" s="18"/>
-    </row>
-    <row r="85" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B85" s="18"/>
-    </row>
-    <row r="86" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B84" s="16"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B85" s="16"/>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B86" s="18"/>
     </row>
-    <row r="87" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B87" s="16"/>
-    </row>
-    <row r="88" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B87" s="18"/>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B88" s="18"/>
     </row>
-    <row r="89" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B89" s="18"/>
-    </row>
-    <row r="90" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B89" s="16"/>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B90" s="18"/>
     </row>
-    <row r="91" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B91" s="18"/>
     </row>
-    <row r="92" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B92" s="18"/>
-      <c r="C92" s="13"/>
-    </row>
-    <row r="93" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B93" s="16"/>
-    </row>
-    <row r="94" spans="2:3" x14ac:dyDescent="0.2">
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B93" s="18"/>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B94" s="18"/>
-    </row>
-    <row r="95" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B95" s="18"/>
-    </row>
-    <row r="96" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C94" s="13"/>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B95" s="16"/>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B96" s="18"/>
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.2">
@@ -3003,7 +3043,13 @@
       <c r="B99" s="18"/>
     </row>
     <row r="100" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B100" s="16"/>
+      <c r="B100" s="18"/>
+    </row>
+    <row r="101" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B101" s="18"/>
+    </row>
+    <row r="102" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B102" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>